<commit_message>
Supplier BOM top board formatting
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/Supplier BOM_Top (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/Supplier BOM_Top (20 Boards).xlsx
@@ -15,21 +15,11 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="389">
   <si>
     <t>Component list</t>
   </si>
@@ -490,18 +480,9 @@
     <t>SOD-123W</t>
   </si>
   <si>
-    <t>0685H9150-01</t>
-  </si>
-  <si>
     <t>MPZ1608S121ATDH5</t>
   </si>
   <si>
-    <t>MC-318</t>
-  </si>
-  <si>
-    <t>5520425-2</t>
-  </si>
-  <si>
     <t>M55-7012642R</t>
   </si>
   <si>
@@ -565,12 +546,6 @@
     <t>SOT-23-6</t>
   </si>
   <si>
-    <t>ISO7741QDBQQ1</t>
-  </si>
-  <si>
-    <t>MAX14850ASE+</t>
-  </si>
-  <si>
     <t>SN74LVTH125PWR</t>
   </si>
   <si>
@@ -595,12 +570,6 @@
     <t>CC0603KRX7R9BB823</t>
   </si>
   <si>
-    <t>08051C224K4T2A</t>
-  </si>
-  <si>
-    <t>CGA3E2X7R2A223K080AA</t>
-  </si>
-  <si>
     <t>CL05B104KB54PNC</t>
   </si>
   <si>
@@ -625,15 +594,9 @@
     <t>CL10B102KC8NNNC</t>
   </si>
   <si>
-    <t>PMEG3010ER,115</t>
-  </si>
-  <si>
     <t>XZVG68W-2</t>
   </si>
   <si>
-    <t>BSC072N08NS5ATMA1</t>
-  </si>
-  <si>
     <t>RC0603JR-075K1L</t>
   </si>
   <si>
@@ -673,9 +636,6 @@
     <t>RC0603FR-07105KL</t>
   </si>
   <si>
-    <t>RT0603FRE07127KL</t>
-  </si>
-  <si>
     <t>RC0603JR-07100KL</t>
   </si>
   <si>
@@ -694,12 +654,6 @@
     <t>RC0603FR-0710KL</t>
   </si>
   <si>
-    <t>NCP708MU330TAG</t>
-  </si>
-  <si>
-    <t>LM43603PWPR</t>
-  </si>
-  <si>
     <t>MC34063ADR</t>
   </si>
   <si>
@@ -1016,9 +970,6 @@
   </si>
   <si>
     <t>IC</t>
-  </si>
-  <si>
-    <t>CRH2512FR033E04Z</t>
   </si>
   <si>
     <t>0603WAF1201T5E</t>
@@ -1327,6 +1278,48 @@
   </si>
   <si>
     <t>XKB Connectivity</t>
+  </si>
+  <si>
+    <t>CC0805KKX7R0BB224</t>
+  </si>
+  <si>
+    <t>TCC0603X7R223K101CT</t>
+  </si>
+  <si>
+    <t>CC0402KRX7R0BB102</t>
+  </si>
+  <si>
+    <t>PMEG3010EP,115</t>
+  </si>
+  <si>
+    <t>12D2150E</t>
+  </si>
+  <si>
+    <t>MC-318FB</t>
+  </si>
+  <si>
+    <t>5520425-3</t>
+  </si>
+  <si>
+    <t>AO4882-MS</t>
+  </si>
+  <si>
+    <t>LR2512-22R033F4</t>
+  </si>
+  <si>
+    <t>ARG03FTC1273</t>
+  </si>
+  <si>
+    <t>TLV75733PDBVR</t>
+  </si>
+  <si>
+    <t>BD9876AEFJ-E2</t>
+  </si>
+  <si>
+    <t>ISO7221ADR</t>
+  </si>
+  <si>
+    <t>ISO6761FDWR</t>
   </si>
 </sst>
 </file>
@@ -1794,7 +1787,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1958,9 +1951,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="17" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2083,6 +2073,51 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2450,10 +2485,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
     </row>
     <row r="2" spans="1:12" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
@@ -2464,7 +2499,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="54" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -2482,14 +2517,14 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="55" t="s">
-        <v>332</v>
+        <v>319</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="102"/>
+      <c r="L3" s="101"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
@@ -2500,14 +2535,14 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="56" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="61"/>
-      <c r="L4" s="103"/>
+      <c r="L4" s="102"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
@@ -2523,7 +2558,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="61"/>
-      <c r="L5" s="103"/>
+      <c r="L5" s="102"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
@@ -2537,7 +2572,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="61"/>
-      <c r="L6" s="103"/>
+      <c r="L6" s="102"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
@@ -2551,7 +2586,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="103"/>
+      <c r="L7" s="102"/>
     </row>
     <row r="8" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="1"/>
@@ -2565,7 +2600,7 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="103"/>
+      <c r="L8" s="102"/>
     </row>
     <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1"/>
@@ -2573,7 +2608,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>7</v>
@@ -2585,22 +2620,22 @@
         <v>141</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="K9" s="31" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="L9" s="31" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2610,7 +2645,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>8</v>
@@ -2619,16 +2654,16 @@
         <v>68</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="G10" s="38" t="s">
         <v>142</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="J10" s="37">
         <v>1</v>
@@ -2645,36 +2680,36 @@
         <f t="shared" ref="B11:B45" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="72" t="s">
-        <v>316</v>
-      </c>
-      <c r="D11" s="73" t="s">
-        <v>374</v>
-      </c>
-      <c r="E11" s="74" t="s">
+      <c r="C11" s="71" t="s">
+        <v>304</v>
+      </c>
+      <c r="D11" s="72" t="s">
+        <v>361</v>
+      </c>
+      <c r="E11" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="73" t="s">
+      <c r="F11" s="72" t="s">
         <v>143</v>
       </c>
-      <c r="G11" s="74" t="s">
-        <v>182</v>
-      </c>
-      <c r="H11" s="73" t="s">
-        <v>228</v>
-      </c>
-      <c r="I11" s="74" t="s">
-        <v>262</v>
-      </c>
-      <c r="J11" s="73">
+      <c r="G11" s="73" t="s">
+        <v>177</v>
+      </c>
+      <c r="H11" s="72" t="s">
+        <v>216</v>
+      </c>
+      <c r="I11" s="73" t="s">
+        <v>250</v>
+      </c>
+      <c r="J11" s="72">
         <v>15</v>
       </c>
-      <c r="K11" s="75">
+      <c r="K11" s="74">
         <f>J11*20</f>
         <v>300</v>
       </c>
-      <c r="L11" s="75" t="s">
-        <v>373</v>
+      <c r="L11" s="74" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2684,10 +2719,10 @@
         <v>3</v>
       </c>
       <c r="C12" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>370</v>
+        <v>357</v>
       </c>
       <c r="E12" s="38" t="s">
         <v>70</v>
@@ -2696,22 +2731,22 @@
         <v>144</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>263</v>
-      </c>
-      <c r="J12" s="76">
+        <v>251</v>
+      </c>
+      <c r="J12" s="75">
         <v>2</v>
       </c>
       <c r="K12" s="41">
         <f t="shared" ref="K12:K71" si="1">J12*20</f>
         <v>40</v>
       </c>
-      <c r="L12" s="68"/>
+      <c r="L12" s="67"/>
     </row>
     <row r="13" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="1"/>
@@ -2720,10 +2755,10 @@
         <v>4</v>
       </c>
       <c r="C13" s="59" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D13" s="39" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="E13" s="40" t="s">
         <v>71</v>
@@ -2732,22 +2767,22 @@
         <v>144</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="I13" s="40" t="s">
-        <v>264</v>
-      </c>
-      <c r="J13" s="77">
+        <v>252</v>
+      </c>
+      <c r="J13" s="76">
         <v>1</v>
       </c>
       <c r="K13" s="42">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L13" s="69"/>
+      <c r="L13" s="68"/>
     </row>
     <row r="14" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1"/>
@@ -2756,10 +2791,10 @@
         <v>5</v>
       </c>
       <c r="C14" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="E14" s="38" t="s">
         <v>72</v>
@@ -2768,13 +2803,13 @@
         <v>143</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="J14" s="37">
         <v>8</v>
@@ -2783,7 +2818,7 @@
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="L14" s="68"/>
+      <c r="L14" s="67"/>
     </row>
     <row r="15" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1"/>
@@ -2792,10 +2827,10 @@
         <v>6</v>
       </c>
       <c r="C15" s="59" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D15" s="39" t="s">
-        <v>369</v>
+        <v>356</v>
       </c>
       <c r="E15" s="40" t="s">
         <v>73</v>
@@ -2804,22 +2839,22 @@
         <v>143</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I15" s="40" t="s">
-        <v>266</v>
-      </c>
-      <c r="J15" s="77">
+        <v>254</v>
+      </c>
+      <c r="J15" s="76">
         <v>3</v>
       </c>
       <c r="K15" s="42">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="L15" s="69"/>
+      <c r="L15" s="68"/>
     </row>
     <row r="16" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1"/>
@@ -2828,25 +2863,25 @@
         <v>7</v>
       </c>
       <c r="C16" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>368</v>
+        <v>355</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>367</v>
+        <v>354</v>
       </c>
       <c r="F16" s="37" t="s">
         <v>143</v>
       </c>
-      <c r="G16" s="87" t="s">
-        <v>345</v>
-      </c>
-      <c r="H16" s="76" t="s">
-        <v>231</v>
+      <c r="G16" s="86" t="s">
+        <v>332</v>
+      </c>
+      <c r="H16" s="75" t="s">
+        <v>219</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="J16" s="37">
         <v>6</v>
@@ -2855,7 +2890,7 @@
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="L16" s="68"/>
+      <c r="L16" s="67"/>
     </row>
     <row r="17" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1"/>
@@ -2864,7 +2899,7 @@
         <v>8</v>
       </c>
       <c r="C17" s="59" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>9</v>
@@ -2876,13 +2911,13 @@
         <v>143</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I17" s="40" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="J17" s="39">
         <v>1</v>
@@ -2899,35 +2934,35 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="88" t="s">
-        <v>316</v>
-      </c>
-      <c r="D18" s="89" t="s">
-        <v>336</v>
-      </c>
-      <c r="E18" s="90" t="s">
+      <c r="C18" s="87" t="s">
+        <v>304</v>
+      </c>
+      <c r="D18" s="88" t="s">
+        <v>323</v>
+      </c>
+      <c r="E18" s="89" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="89" t="s">
+      <c r="F18" s="88" t="s">
         <v>145</v>
       </c>
-      <c r="G18" s="90" t="s">
-        <v>188</v>
-      </c>
-      <c r="H18" s="89" t="s">
-        <v>232</v>
-      </c>
-      <c r="I18" s="90" t="s">
-        <v>269</v>
-      </c>
-      <c r="J18" s="89">
+      <c r="G18" s="103" t="s">
+        <v>375</v>
+      </c>
+      <c r="H18" s="88" t="s">
+        <v>220</v>
+      </c>
+      <c r="I18" s="89" t="s">
+        <v>257</v>
+      </c>
+      <c r="J18" s="88">
         <v>8</v>
       </c>
-      <c r="K18" s="83">
+      <c r="K18" s="82">
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="L18" s="83"/>
+      <c r="L18" s="82"/>
     </row>
     <row r="19" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1"/>
@@ -2935,35 +2970,35 @@
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="91" t="s">
-        <v>316</v>
-      </c>
-      <c r="D19" s="92" t="s">
+      <c r="C19" s="90" t="s">
+        <v>304</v>
+      </c>
+      <c r="D19" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="93" t="s">
+      <c r="E19" s="92" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="92" t="s">
+      <c r="F19" s="91" t="s">
         <v>143</v>
       </c>
-      <c r="G19" s="93" t="s">
-        <v>189</v>
-      </c>
-      <c r="H19" s="92" t="s">
-        <v>233</v>
-      </c>
-      <c r="I19" s="93" t="s">
-        <v>270</v>
-      </c>
-      <c r="J19" s="92">
+      <c r="G19" s="104" t="s">
+        <v>376</v>
+      </c>
+      <c r="H19" s="91" t="s">
+        <v>221</v>
+      </c>
+      <c r="I19" s="92" t="s">
+        <v>258</v>
+      </c>
+      <c r="J19" s="91">
         <v>1</v>
       </c>
-      <c r="K19" s="94">
+      <c r="K19" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L19" s="94"/>
+      <c r="L19" s="93"/>
     </row>
     <row r="20" spans="1:12" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="1"/>
@@ -2971,35 +3006,35 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="88" t="s">
-        <v>316</v>
-      </c>
-      <c r="D20" s="89" t="s">
+      <c r="C20" s="87" t="s">
+        <v>304</v>
+      </c>
+      <c r="D20" s="88" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="90" t="s">
+      <c r="E20" s="89" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G20" s="89" t="s">
+      <c r="F20" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G20" s="88" t="s">
         <v>146</v>
       </c>
-      <c r="H20" s="89" t="s">
-        <v>234</v>
-      </c>
-      <c r="I20" s="90" t="s">
-        <v>261</v>
-      </c>
-      <c r="J20" s="89">
+      <c r="H20" s="88" t="s">
+        <v>222</v>
+      </c>
+      <c r="I20" s="89" t="s">
+        <v>249</v>
+      </c>
+      <c r="J20" s="88">
         <v>1</v>
       </c>
-      <c r="K20" s="83">
+      <c r="K20" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L20" s="83"/>
+      <c r="L20" s="82"/>
     </row>
     <row r="21" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
@@ -3007,35 +3042,35 @@
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="91" t="s">
-        <v>316</v>
-      </c>
-      <c r="D21" s="92" t="s">
+      <c r="C21" s="90" t="s">
+        <v>304</v>
+      </c>
+      <c r="D21" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="93" t="s">
+      <c r="E21" s="92" t="s">
         <v>78</v>
       </c>
-      <c r="F21" s="92" t="s">
+      <c r="F21" s="91" t="s">
         <v>144</v>
       </c>
-      <c r="G21" s="93" t="s">
-        <v>190</v>
-      </c>
-      <c r="H21" s="92" t="s">
-        <v>228</v>
-      </c>
-      <c r="I21" s="93" t="s">
-        <v>271</v>
-      </c>
-      <c r="J21" s="92">
+      <c r="G21" s="92" t="s">
+        <v>183</v>
+      </c>
+      <c r="H21" s="91" t="s">
+        <v>216</v>
+      </c>
+      <c r="I21" s="92" t="s">
+        <v>259</v>
+      </c>
+      <c r="J21" s="91">
         <v>2</v>
       </c>
-      <c r="K21" s="94">
+      <c r="K21" s="93">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L21" s="94"/>
+      <c r="L21" s="93"/>
     </row>
     <row r="22" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
@@ -3044,7 +3079,7 @@
         <v>13</v>
       </c>
       <c r="C22" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D22" s="37" t="s">
         <v>13</v>
@@ -3056,13 +3091,13 @@
         <v>143</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="J22" s="37">
         <v>1</v>
@@ -3080,10 +3115,10 @@
         <v>14</v>
       </c>
       <c r="C23" s="59" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D23" s="39" t="s">
-        <v>342</v>
+        <v>329</v>
       </c>
       <c r="E23" s="40" t="s">
         <v>80</v>
@@ -3092,13 +3127,13 @@
         <v>143</v>
       </c>
       <c r="G23" s="40" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="H23" s="39" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="I23" s="40" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="J23" s="39">
         <v>1</v>
@@ -3107,7 +3142,7 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L23" s="69"/>
+      <c r="L23" s="68"/>
     </row>
     <row r="24" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
@@ -3116,7 +3151,7 @@
         <v>15</v>
       </c>
       <c r="C24" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D24" s="37" t="s">
         <v>14</v>
@@ -3127,14 +3162,14 @@
       <c r="F24" s="37" t="s">
         <v>144</v>
       </c>
-      <c r="G24" s="62">
-        <v>885012205080</v>
+      <c r="G24" s="105" t="s">
+        <v>377</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="J24" s="37">
         <v>1</v>
@@ -3152,7 +3187,7 @@
         <v>16</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D25" s="39" t="s">
         <v>15</v>
@@ -3164,13 +3199,13 @@
         <v>143</v>
       </c>
       <c r="G25" s="40" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="J25" s="39">
         <v>1</v>
@@ -3187,35 +3222,35 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="88" t="s">
-        <v>316</v>
-      </c>
-      <c r="D26" s="89" t="s">
+      <c r="C26" s="87" t="s">
+        <v>304</v>
+      </c>
+      <c r="D26" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="E26" s="95" t="s">
-        <v>344</v>
-      </c>
-      <c r="F26" s="89" t="s">
+      <c r="E26" s="94" t="s">
+        <v>331</v>
+      </c>
+      <c r="F26" s="88" t="s">
         <v>143</v>
       </c>
-      <c r="G26" s="95" t="s">
-        <v>366</v>
-      </c>
-      <c r="H26" s="96" t="s">
-        <v>249</v>
-      </c>
-      <c r="I26" s="95" t="s">
+      <c r="G26" s="94" t="s">
         <v>353</v>
       </c>
-      <c r="J26" s="89">
+      <c r="H26" s="95" t="s">
+        <v>237</v>
+      </c>
+      <c r="I26" s="94" t="s">
+        <v>340</v>
+      </c>
+      <c r="J26" s="88">
         <v>1</v>
       </c>
-      <c r="K26" s="83">
+      <c r="K26" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L26" s="68"/>
+      <c r="L26" s="67"/>
     </row>
     <row r="27" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1"/>
@@ -3223,35 +3258,35 @@
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="91" t="s">
-        <v>316</v>
-      </c>
-      <c r="D27" s="92" t="s">
-        <v>352</v>
-      </c>
-      <c r="E27" s="93" t="s">
+      <c r="C27" s="90" t="s">
+        <v>304</v>
+      </c>
+      <c r="D27" s="91" t="s">
+        <v>339</v>
+      </c>
+      <c r="E27" s="92" t="s">
         <v>83</v>
       </c>
-      <c r="F27" s="92" t="s">
+      <c r="F27" s="91" t="s">
         <v>147</v>
       </c>
-      <c r="G27" s="93" t="s">
-        <v>194</v>
-      </c>
-      <c r="H27" s="92" t="s">
-        <v>231</v>
-      </c>
-      <c r="I27" s="93" t="s">
-        <v>275</v>
-      </c>
-      <c r="J27" s="92">
+      <c r="G27" s="92" t="s">
+        <v>187</v>
+      </c>
+      <c r="H27" s="91" t="s">
+        <v>219</v>
+      </c>
+      <c r="I27" s="92" t="s">
+        <v>263</v>
+      </c>
+      <c r="J27" s="91">
         <v>1</v>
       </c>
-      <c r="K27" s="94">
+      <c r="K27" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L27" s="71"/>
+      <c r="L27" s="70"/>
     </row>
     <row r="28" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1"/>
@@ -3260,7 +3295,7 @@
         <v>19</v>
       </c>
       <c r="C28" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D28" s="37" t="s">
         <v>17</v>
@@ -3272,13 +3307,13 @@
         <v>148</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="J28" s="37">
         <v>1</v>
@@ -3296,7 +3331,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="59" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D29" s="39" t="s">
         <v>18</v>
@@ -3305,16 +3340,16 @@
         <v>85</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="G29" s="39" t="s">
         <v>149</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="J29" s="39">
         <v>1</v>
@@ -3332,7 +3367,7 @@
         <v>21</v>
       </c>
       <c r="C30" s="60" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D30" s="37" t="s">
         <v>19</v>
@@ -3344,13 +3379,13 @@
         <v>143</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="H30" s="37" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I30" s="38" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="J30" s="37">
         <v>1</v>
@@ -3367,35 +3402,35 @@
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="91" t="s">
-        <v>316</v>
-      </c>
-      <c r="D31" s="92" t="s">
+      <c r="C31" s="90" t="s">
+        <v>304</v>
+      </c>
+      <c r="D31" s="91" t="s">
         <v>20</v>
       </c>
-      <c r="E31" s="93" t="s">
+      <c r="E31" s="92" t="s">
         <v>87</v>
       </c>
-      <c r="F31" s="92" t="s">
+      <c r="F31" s="91" t="s">
         <v>143</v>
       </c>
-      <c r="G31" s="93" t="s">
-        <v>197</v>
-      </c>
-      <c r="H31" s="92" t="s">
-        <v>228</v>
-      </c>
-      <c r="I31" s="93" t="s">
-        <v>279</v>
-      </c>
-      <c r="J31" s="92">
+      <c r="G31" s="92" t="s">
+        <v>190</v>
+      </c>
+      <c r="H31" s="91" t="s">
+        <v>216</v>
+      </c>
+      <c r="I31" s="92" t="s">
+        <v>267</v>
+      </c>
+      <c r="J31" s="91">
         <v>4</v>
       </c>
-      <c r="K31" s="94">
+      <c r="K31" s="93">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L31" s="94"/>
+      <c r="L31" s="93"/>
     </row>
     <row r="32" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="1"/>
@@ -3403,35 +3438,35 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="88" t="s">
-        <v>317</v>
-      </c>
-      <c r="D32" s="89" t="s">
+      <c r="C32" s="87" t="s">
+        <v>305</v>
+      </c>
+      <c r="D32" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="90" t="s">
+      <c r="E32" s="89" t="s">
         <v>88</v>
       </c>
-      <c r="F32" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G32" s="90" t="s">
+      <c r="F32" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G32" s="89" t="s">
         <v>150</v>
       </c>
-      <c r="H32" s="89" t="s">
-        <v>237</v>
-      </c>
-      <c r="I32" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J32" s="89">
+      <c r="H32" s="88" t="s">
+        <v>225</v>
+      </c>
+      <c r="I32" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J32" s="88">
         <v>1</v>
       </c>
-      <c r="K32" s="83">
+      <c r="K32" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L32" s="83"/>
+      <c r="L32" s="82"/>
     </row>
     <row r="33" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="1"/>
@@ -3439,35 +3474,35 @@
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
-      <c r="C33" s="91" t="s">
-        <v>317</v>
-      </c>
-      <c r="D33" s="92" t="s">
+      <c r="C33" s="90" t="s">
+        <v>305</v>
+      </c>
+      <c r="D33" s="91" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="93" t="s">
+      <c r="E33" s="92" t="s">
         <v>89</v>
       </c>
-      <c r="F33" s="92" t="s">
+      <c r="F33" s="91" t="s">
         <v>151</v>
       </c>
-      <c r="G33" s="93" t="s">
-        <v>280</v>
-      </c>
-      <c r="H33" s="92" t="s">
-        <v>238</v>
-      </c>
-      <c r="I33" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J33" s="92">
+      <c r="G33" s="92" t="s">
+        <v>268</v>
+      </c>
+      <c r="H33" s="91" t="s">
+        <v>226</v>
+      </c>
+      <c r="I33" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J33" s="91">
         <v>1</v>
       </c>
-      <c r="K33" s="94">
+      <c r="K33" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L33" s="94"/>
+      <c r="L33" s="93"/>
     </row>
     <row r="34" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
@@ -3475,35 +3510,35 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="88" t="s">
-        <v>317</v>
-      </c>
-      <c r="D34" s="89" t="s">
-        <v>371</v>
-      </c>
-      <c r="E34" s="90" t="s">
+      <c r="C34" s="87" t="s">
+        <v>305</v>
+      </c>
+      <c r="D34" s="88" t="s">
+        <v>358</v>
+      </c>
+      <c r="E34" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="F34" s="89" t="s">
+      <c r="F34" s="88" t="s">
         <v>151</v>
       </c>
-      <c r="G34" s="90" t="s">
-        <v>281</v>
-      </c>
-      <c r="H34" s="89" t="s">
-        <v>238</v>
-      </c>
-      <c r="I34" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J34" s="89">
+      <c r="G34" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="H34" s="88" t="s">
+        <v>226</v>
+      </c>
+      <c r="I34" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J34" s="88">
         <v>2</v>
       </c>
-      <c r="K34" s="83">
+      <c r="K34" s="82">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L34" s="70"/>
+      <c r="L34" s="69"/>
     </row>
     <row r="35" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="1"/>
@@ -3511,38 +3546,38 @@
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
-      <c r="C35" s="78" t="s">
-        <v>317</v>
-      </c>
-      <c r="D35" s="79" t="s">
-        <v>354</v>
-      </c>
-      <c r="E35" s="80" t="s">
+      <c r="C35" s="77" t="s">
+        <v>305</v>
+      </c>
+      <c r="D35" s="78" t="s">
+        <v>341</v>
+      </c>
+      <c r="E35" s="79" t="s">
         <v>91</v>
       </c>
-      <c r="F35" s="79" t="s">
+      <c r="F35" s="78" t="s">
         <v>152</v>
       </c>
-      <c r="G35" s="80" t="s">
-        <v>198</v>
-      </c>
-      <c r="H35" s="79" t="s">
-        <v>239</v>
-      </c>
-      <c r="I35" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="J35" s="81">
+      <c r="G35" s="107" t="s">
+        <v>378</v>
+      </c>
+      <c r="H35" s="78" t="s">
+        <v>227</v>
+      </c>
+      <c r="I35" s="79" t="s">
+        <v>302</v>
+      </c>
+      <c r="J35" s="80">
         <v>8</v>
       </c>
-      <c r="K35" s="82">
+      <c r="K35" s="81">
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="L35" s="75" t="s">
-        <v>355</v>
-      </c>
-      <c r="O35" s="100"/>
+      <c r="L35" s="74" t="s">
+        <v>342</v>
+      </c>
+      <c r="O35" s="99"/>
     </row>
     <row r="36" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1"/>
@@ -3550,35 +3585,35 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="88" t="s">
-        <v>319</v>
-      </c>
-      <c r="D36" s="89" t="s">
+      <c r="C36" s="87" t="s">
+        <v>307</v>
+      </c>
+      <c r="D36" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="E36" s="90" t="s">
+      <c r="E36" s="89" t="s">
         <v>92</v>
       </c>
-      <c r="F36" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G36" s="90" t="s">
-        <v>153</v>
-      </c>
-      <c r="H36" s="89" t="s">
-        <v>240</v>
-      </c>
-      <c r="I36" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J36" s="89">
+      <c r="F36" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G36" s="108" t="s">
+        <v>379</v>
+      </c>
+      <c r="H36" s="88" t="s">
+        <v>228</v>
+      </c>
+      <c r="I36" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J36" s="88">
         <v>1</v>
       </c>
-      <c r="K36" s="83">
+      <c r="K36" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L36" s="83"/>
+      <c r="L36" s="82"/>
     </row>
     <row r="37" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="1"/>
@@ -3586,35 +3621,35 @@
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="91" t="s">
-        <v>318</v>
-      </c>
-      <c r="D37" s="92" t="s">
+      <c r="C37" s="90" t="s">
+        <v>306</v>
+      </c>
+      <c r="D37" s="91" t="s">
         <v>24</v>
       </c>
-      <c r="E37" s="93" t="s">
+      <c r="E37" s="92" t="s">
         <v>93</v>
       </c>
-      <c r="F37" s="92" t="s">
-        <v>309</v>
-      </c>
-      <c r="G37" s="93" t="s">
-        <v>154</v>
-      </c>
-      <c r="H37" s="92" t="s">
-        <v>233</v>
-      </c>
-      <c r="I37" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J37" s="92">
+      <c r="F37" s="91" t="s">
+        <v>297</v>
+      </c>
+      <c r="G37" s="92" t="s">
+        <v>153</v>
+      </c>
+      <c r="H37" s="91" t="s">
+        <v>221</v>
+      </c>
+      <c r="I37" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J37" s="91">
         <v>4</v>
       </c>
-      <c r="K37" s="94">
+      <c r="K37" s="93">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L37" s="94"/>
+      <c r="L37" s="93"/>
     </row>
     <row r="38" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="1"/>
@@ -3622,35 +3657,35 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="88" t="s">
-        <v>320</v>
-      </c>
-      <c r="D38" s="89" t="s">
+      <c r="C38" s="87" t="s">
+        <v>308</v>
+      </c>
+      <c r="D38" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="E38" s="90" t="s">
+      <c r="E38" s="89" t="s">
         <v>94</v>
       </c>
-      <c r="F38" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G38" s="90" t="s">
-        <v>155</v>
-      </c>
-      <c r="H38" s="89" t="s">
-        <v>241</v>
-      </c>
-      <c r="I38" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J38" s="89">
+      <c r="F38" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G38" s="109" t="s">
+        <v>380</v>
+      </c>
+      <c r="H38" s="88" t="s">
+        <v>229</v>
+      </c>
+      <c r="I38" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J38" s="88">
         <v>1</v>
       </c>
-      <c r="K38" s="83">
+      <c r="K38" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L38" s="70"/>
+      <c r="L38" s="69"/>
     </row>
     <row r="39" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="1"/>
@@ -3658,35 +3693,35 @@
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="91" t="s">
-        <v>320</v>
-      </c>
-      <c r="D39" s="92" t="s">
+      <c r="C39" s="90" t="s">
+        <v>308</v>
+      </c>
+      <c r="D39" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="E39" s="93" t="s">
+      <c r="E39" s="92" t="s">
         <v>95</v>
       </c>
-      <c r="F39" s="92" t="s">
-        <v>308</v>
-      </c>
-      <c r="G39" s="93" t="s">
-        <v>156</v>
-      </c>
-      <c r="H39" s="92" t="s">
-        <v>242</v>
-      </c>
-      <c r="I39" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J39" s="92">
+      <c r="F39" s="91" t="s">
+        <v>296</v>
+      </c>
+      <c r="G39" s="110" t="s">
+        <v>381</v>
+      </c>
+      <c r="H39" s="91" t="s">
+        <v>230</v>
+      </c>
+      <c r="I39" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J39" s="91">
         <v>2</v>
       </c>
-      <c r="K39" s="94">
+      <c r="K39" s="93">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L39" s="71"/>
+      <c r="L39" s="70"/>
     </row>
     <row r="40" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="1"/>
@@ -3694,35 +3729,35 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="88" t="s">
-        <v>321</v>
-      </c>
-      <c r="D40" s="89" t="s">
+      <c r="C40" s="87" t="s">
+        <v>309</v>
+      </c>
+      <c r="D40" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="E40" s="90" t="s">
+      <c r="E40" s="89" t="s">
         <v>96</v>
       </c>
-      <c r="F40" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G40" s="90" t="s">
-        <v>157</v>
-      </c>
-      <c r="H40" s="89" t="s">
-        <v>243</v>
-      </c>
-      <c r="I40" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J40" s="89">
+      <c r="F40" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G40" s="89" t="s">
+        <v>154</v>
+      </c>
+      <c r="H40" s="88" t="s">
+        <v>231</v>
+      </c>
+      <c r="I40" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J40" s="88">
         <v>1</v>
       </c>
-      <c r="K40" s="83">
+      <c r="K40" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L40" s="83"/>
+      <c r="L40" s="82"/>
     </row>
     <row r="41" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="1"/>
@@ -3730,68 +3765,68 @@
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="91" t="s">
-        <v>321</v>
-      </c>
-      <c r="D41" s="92" t="s">
+      <c r="C41" s="90" t="s">
+        <v>309</v>
+      </c>
+      <c r="D41" s="91" t="s">
         <v>28</v>
       </c>
-      <c r="E41" s="93" t="s">
+      <c r="E41" s="92" t="s">
         <v>97</v>
       </c>
-      <c r="F41" s="92" t="s">
-        <v>308</v>
-      </c>
-      <c r="G41" s="93" t="s">
-        <v>158</v>
-      </c>
-      <c r="H41" s="92" t="s">
-        <v>244</v>
-      </c>
-      <c r="I41" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J41" s="92">
+      <c r="F41" s="91" t="s">
+        <v>296</v>
+      </c>
+      <c r="G41" s="92" t="s">
+        <v>155</v>
+      </c>
+      <c r="H41" s="91" t="s">
+        <v>232</v>
+      </c>
+      <c r="I41" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J41" s="91">
         <v>1</v>
       </c>
-      <c r="K41" s="94">
+      <c r="K41" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L41" s="94"/>
+      <c r="L41" s="93"/>
     </row>
     <row r="42" spans="1:15" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="1"/>
       <c r="B42" s="53"/>
-      <c r="C42" s="91" t="s">
-        <v>321</v>
-      </c>
-      <c r="D42" s="92" t="s">
-        <v>384</v>
-      </c>
-      <c r="E42" s="93" t="s">
-        <v>386</v>
-      </c>
-      <c r="F42" s="92" t="s">
-        <v>308</v>
-      </c>
-      <c r="G42" s="93" t="s">
-        <v>385</v>
-      </c>
-      <c r="H42" s="92" t="s">
-        <v>387</v>
-      </c>
-      <c r="I42" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J42" s="92">
+      <c r="C42" s="90" t="s">
+        <v>309</v>
+      </c>
+      <c r="D42" s="91" t="s">
+        <v>371</v>
+      </c>
+      <c r="E42" s="92" t="s">
+        <v>373</v>
+      </c>
+      <c r="F42" s="91" t="s">
+        <v>296</v>
+      </c>
+      <c r="G42" s="92" t="s">
+        <v>372</v>
+      </c>
+      <c r="H42" s="91" t="s">
+        <v>374</v>
+      </c>
+      <c r="I42" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J42" s="91">
         <v>1</v>
       </c>
-      <c r="K42" s="94">
+      <c r="K42" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L42" s="94"/>
+      <c r="L42" s="93"/>
     </row>
     <row r="43" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="1"/>
@@ -3799,35 +3834,35 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="88" t="s">
-        <v>318</v>
-      </c>
-      <c r="D43" s="89" t="s">
+      <c r="C43" s="87" t="s">
+        <v>306</v>
+      </c>
+      <c r="D43" s="88" t="s">
         <v>29</v>
       </c>
-      <c r="E43" s="90" t="s">
+      <c r="E43" s="89" t="s">
         <v>98</v>
       </c>
-      <c r="F43" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G43" s="90" t="s">
-        <v>159</v>
-      </c>
-      <c r="H43" s="89" t="s">
-        <v>233</v>
-      </c>
-      <c r="I43" s="90" t="s">
-        <v>282</v>
-      </c>
-      <c r="J43" s="89">
+      <c r="F43" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G43" s="89" t="s">
+        <v>156</v>
+      </c>
+      <c r="H43" s="88" t="s">
+        <v>221</v>
+      </c>
+      <c r="I43" s="89" t="s">
+        <v>270</v>
+      </c>
+      <c r="J43" s="88">
         <v>1</v>
       </c>
-      <c r="K43" s="83">
+      <c r="K43" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L43" s="83"/>
+      <c r="L43" s="82"/>
     </row>
     <row r="44" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="1"/>
@@ -3835,35 +3870,35 @@
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="91" t="s">
-        <v>318</v>
-      </c>
-      <c r="D44" s="92" t="s">
+      <c r="C44" s="90" t="s">
+        <v>306</v>
+      </c>
+      <c r="D44" s="91" t="s">
         <v>30</v>
       </c>
-      <c r="E44" s="93" t="s">
-        <v>358</v>
-      </c>
-      <c r="F44" s="92" t="s">
-        <v>308</v>
-      </c>
-      <c r="G44" s="93" t="s">
-        <v>357</v>
-      </c>
-      <c r="H44" s="92" t="s">
-        <v>347</v>
-      </c>
-      <c r="I44" s="93" t="s">
-        <v>356</v>
-      </c>
-      <c r="J44" s="92">
+      <c r="E44" s="92" t="s">
+        <v>345</v>
+      </c>
+      <c r="F44" s="91" t="s">
+        <v>296</v>
+      </c>
+      <c r="G44" s="92" t="s">
+        <v>344</v>
+      </c>
+      <c r="H44" s="91" t="s">
+        <v>334</v>
+      </c>
+      <c r="I44" s="92" t="s">
+        <v>343</v>
+      </c>
+      <c r="J44" s="91">
         <v>1</v>
       </c>
-      <c r="K44" s="94">
+      <c r="K44" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L44" s="69"/>
+      <c r="L44" s="68"/>
     </row>
     <row r="45" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="1"/>
@@ -3871,35 +3906,35 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="88" t="s">
-        <v>322</v>
-      </c>
-      <c r="D45" s="89" t="s">
+      <c r="C45" s="87" t="s">
+        <v>310</v>
+      </c>
+      <c r="D45" s="88" t="s">
         <v>31</v>
       </c>
-      <c r="E45" s="90" t="s">
+      <c r="E45" s="89" t="s">
         <v>99</v>
       </c>
-      <c r="F45" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G45" s="90" t="s">
-        <v>160</v>
-      </c>
-      <c r="H45" s="89" t="s">
-        <v>245</v>
-      </c>
-      <c r="I45" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J45" s="89">
+      <c r="F45" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G45" s="89" t="s">
+        <v>157</v>
+      </c>
+      <c r="H45" s="88" t="s">
+        <v>233</v>
+      </c>
+      <c r="I45" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J45" s="88">
         <v>1</v>
       </c>
-      <c r="K45" s="83">
+      <c r="K45" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L45" s="83"/>
+      <c r="L45" s="82"/>
     </row>
     <row r="46" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="1"/>
@@ -3907,35 +3942,35 @@
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="91" t="s">
-        <v>322</v>
-      </c>
-      <c r="D46" s="92" t="s">
+      <c r="C46" s="90" t="s">
+        <v>310</v>
+      </c>
+      <c r="D46" s="91" t="s">
         <v>32</v>
       </c>
-      <c r="E46" s="93" t="s">
+      <c r="E46" s="92" t="s">
         <v>100</v>
       </c>
-      <c r="F46" s="92" t="s">
-        <v>161</v>
-      </c>
-      <c r="G46" s="93" t="s">
-        <v>199</v>
-      </c>
-      <c r="H46" s="92" t="s">
-        <v>246</v>
-      </c>
-      <c r="I46" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J46" s="92">
+      <c r="F46" s="91" t="s">
+        <v>158</v>
+      </c>
+      <c r="G46" s="92" t="s">
+        <v>191</v>
+      </c>
+      <c r="H46" s="91" t="s">
+        <v>234</v>
+      </c>
+      <c r="I46" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J46" s="91">
         <v>1</v>
       </c>
-      <c r="K46" s="94">
+      <c r="K46" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L46" s="94"/>
+      <c r="L46" s="93"/>
     </row>
     <row r="47" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="1"/>
@@ -3943,36 +3978,36 @@
         <f t="shared" ref="B47:B90" si="2">ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
-      <c r="C47" s="91" t="s">
-        <v>375</v>
-      </c>
-      <c r="D47" s="92" t="s">
-        <v>314</v>
-      </c>
-      <c r="E47" s="93" t="s">
-        <v>377</v>
-      </c>
-      <c r="F47" s="92" t="s">
-        <v>308</v>
-      </c>
-      <c r="G47" s="93" t="s">
-        <v>378</v>
-      </c>
-      <c r="H47" s="92" t="s">
-        <v>379</v>
-      </c>
-      <c r="I47" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J47" s="92">
+      <c r="C47" s="90" t="s">
+        <v>362</v>
+      </c>
+      <c r="D47" s="91" t="s">
+        <v>302</v>
+      </c>
+      <c r="E47" s="92" t="s">
+        <v>364</v>
+      </c>
+      <c r="F47" s="91" t="s">
+        <v>296</v>
+      </c>
+      <c r="G47" s="92" t="s">
+        <v>365</v>
+      </c>
+      <c r="H47" s="91" t="s">
+        <v>366</v>
+      </c>
+      <c r="I47" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J47" s="91">
         <v>1</v>
       </c>
-      <c r="K47" s="94">
+      <c r="K47" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L47" s="71" t="s">
-        <v>376</v>
+      <c r="L47" s="70" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="48" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3981,35 +4016,35 @@
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="C48" s="88" t="s">
-        <v>320</v>
-      </c>
-      <c r="D48" s="89" t="s">
+      <c r="C48" s="87" t="s">
+        <v>308</v>
+      </c>
+      <c r="D48" s="88" t="s">
         <v>33</v>
       </c>
-      <c r="E48" s="90" t="s">
+      <c r="E48" s="89" t="s">
         <v>101</v>
       </c>
-      <c r="F48" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G48" s="90" t="s">
-        <v>162</v>
-      </c>
-      <c r="H48" s="89" t="s">
-        <v>247</v>
-      </c>
-      <c r="I48" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J48" s="89">
+      <c r="F48" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G48" s="89" t="s">
+        <v>159</v>
+      </c>
+      <c r="H48" s="88" t="s">
+        <v>235</v>
+      </c>
+      <c r="I48" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J48" s="88">
         <v>2</v>
       </c>
-      <c r="K48" s="83">
+      <c r="K48" s="82">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L48" s="83"/>
+      <c r="L48" s="82"/>
     </row>
     <row r="49" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="1"/>
@@ -4017,36 +4052,36 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="C49" s="84" t="s">
-        <v>283</v>
-      </c>
-      <c r="D49" s="85" t="s">
+      <c r="C49" s="83" t="s">
+        <v>271</v>
+      </c>
+      <c r="D49" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="E49" s="86" t="s">
+      <c r="E49" s="85" t="s">
         <v>102</v>
       </c>
-      <c r="F49" s="85" t="s">
-        <v>163</v>
-      </c>
-      <c r="G49" s="86" t="s">
-        <v>314</v>
-      </c>
-      <c r="H49" s="85" t="s">
-        <v>314</v>
-      </c>
-      <c r="I49" s="86" t="s">
-        <v>314</v>
-      </c>
-      <c r="J49" s="85">
+      <c r="F49" s="84" t="s">
+        <v>160</v>
+      </c>
+      <c r="G49" s="85" t="s">
+        <v>302</v>
+      </c>
+      <c r="H49" s="84" t="s">
+        <v>302</v>
+      </c>
+      <c r="I49" s="85" t="s">
+        <v>302</v>
+      </c>
+      <c r="J49" s="84">
         <v>4</v>
       </c>
-      <c r="K49" s="63">
+      <c r="K49" s="62">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L49" s="63" t="s">
-        <v>337</v>
+      <c r="L49" s="62" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -4055,35 +4090,35 @@
         <f t="shared" si="2"/>
         <v>41</v>
       </c>
-      <c r="C50" s="88" t="s">
-        <v>321</v>
-      </c>
-      <c r="D50" s="89" t="s">
+      <c r="C50" s="87" t="s">
+        <v>309</v>
+      </c>
+      <c r="D50" s="88" t="s">
         <v>35</v>
       </c>
-      <c r="E50" s="90" t="s">
+      <c r="E50" s="89" t="s">
         <v>103</v>
       </c>
-      <c r="F50" s="89" t="s">
-        <v>164</v>
-      </c>
-      <c r="G50" s="90">
+      <c r="F50" s="88" t="s">
+        <v>161</v>
+      </c>
+      <c r="G50" s="89">
         <v>61300211121</v>
       </c>
-      <c r="H50" s="89" t="s">
-        <v>235</v>
-      </c>
-      <c r="I50" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J50" s="89">
+      <c r="H50" s="88" t="s">
+        <v>223</v>
+      </c>
+      <c r="I50" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J50" s="88">
         <v>4</v>
       </c>
-      <c r="K50" s="83">
+      <c r="K50" s="82">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L50" s="83"/>
+      <c r="L50" s="82"/>
     </row>
     <row r="51" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="1"/>
@@ -4091,35 +4126,35 @@
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
-      <c r="C51" s="91" t="s">
-        <v>323</v>
-      </c>
-      <c r="D51" s="92" t="s">
-        <v>349</v>
-      </c>
-      <c r="E51" s="93" t="s">
+      <c r="C51" s="90" t="s">
+        <v>311</v>
+      </c>
+      <c r="D51" s="91" t="s">
+        <v>336</v>
+      </c>
+      <c r="E51" s="92" t="s">
         <v>104</v>
       </c>
-      <c r="F51" s="92" t="s">
-        <v>165</v>
-      </c>
-      <c r="G51" s="93" t="s">
-        <v>200</v>
-      </c>
-      <c r="H51" s="92" t="s">
-        <v>248</v>
-      </c>
-      <c r="I51" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J51" s="92">
+      <c r="F51" s="91" t="s">
+        <v>162</v>
+      </c>
+      <c r="G51" s="111" t="s">
+        <v>382</v>
+      </c>
+      <c r="H51" s="91" t="s">
+        <v>236</v>
+      </c>
+      <c r="I51" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J51" s="91">
         <v>4</v>
       </c>
-      <c r="K51" s="94">
+      <c r="K51" s="93">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L51" s="94"/>
+      <c r="L51" s="93"/>
     </row>
     <row r="52" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="1"/>
@@ -4127,35 +4162,35 @@
         <f t="shared" si="2"/>
         <v>43</v>
       </c>
-      <c r="C52" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D52" s="89" t="s">
+      <c r="C52" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D52" s="88" t="s">
         <v>36</v>
       </c>
-      <c r="E52" s="90" t="s">
+      <c r="E52" s="89" t="s">
         <v>105</v>
       </c>
-      <c r="F52" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G52" s="90" t="s">
-        <v>201</v>
-      </c>
-      <c r="H52" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="I52" s="90" t="s">
-        <v>284</v>
-      </c>
-      <c r="J52" s="89">
+      <c r="F52" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G52" s="89" t="s">
+        <v>192</v>
+      </c>
+      <c r="H52" s="88" t="s">
+        <v>217</v>
+      </c>
+      <c r="I52" s="89" t="s">
+        <v>272</v>
+      </c>
+      <c r="J52" s="88">
         <v>2</v>
       </c>
-      <c r="K52" s="83">
+      <c r="K52" s="82">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L52" s="83"/>
+      <c r="L52" s="82"/>
     </row>
     <row r="53" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="1"/>
@@ -4163,35 +4198,35 @@
         <f t="shared" si="2"/>
         <v>44</v>
       </c>
-      <c r="C53" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D53" s="92" t="s">
+      <c r="C53" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D53" s="91" t="s">
         <v>37</v>
       </c>
-      <c r="E53" s="93" t="s">
+      <c r="E53" s="92" t="s">
         <v>106</v>
       </c>
-      <c r="F53" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G53" s="93" t="s">
-        <v>202</v>
-      </c>
-      <c r="H53" s="92" t="s">
-        <v>229</v>
-      </c>
-      <c r="I53" s="93" t="s">
-        <v>285</v>
-      </c>
-      <c r="J53" s="92">
+      <c r="F53" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G53" s="92" t="s">
+        <v>193</v>
+      </c>
+      <c r="H53" s="91" t="s">
+        <v>217</v>
+      </c>
+      <c r="I53" s="92" t="s">
+        <v>273</v>
+      </c>
+      <c r="J53" s="91">
         <v>1</v>
       </c>
-      <c r="K53" s="94">
+      <c r="K53" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L53" s="94"/>
+      <c r="L53" s="93"/>
     </row>
     <row r="54" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="1"/>
@@ -4199,35 +4234,35 @@
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="C54" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D54" s="89" t="s">
+      <c r="C54" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D54" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="E54" s="90" t="s">
+      <c r="E54" s="89" t="s">
         <v>107</v>
       </c>
-      <c r="F54" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G54" s="90" t="s">
-        <v>203</v>
-      </c>
-      <c r="H54" s="89" t="s">
-        <v>249</v>
-      </c>
-      <c r="I54" s="90" t="s">
-        <v>286</v>
-      </c>
-      <c r="J54" s="89">
+      <c r="F54" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G54" s="89" t="s">
+        <v>194</v>
+      </c>
+      <c r="H54" s="88" t="s">
+        <v>237</v>
+      </c>
+      <c r="I54" s="89" t="s">
+        <v>274</v>
+      </c>
+      <c r="J54" s="88">
         <v>1</v>
       </c>
-      <c r="K54" s="83">
+      <c r="K54" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L54" s="83"/>
+      <c r="L54" s="82"/>
     </row>
     <row r="55" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="1"/>
@@ -4235,35 +4270,35 @@
         <f t="shared" si="2"/>
         <v>46</v>
       </c>
-      <c r="C55" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D55" s="92" t="s">
+      <c r="C55" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D55" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="E55" s="93" t="s">
+      <c r="E55" s="92" t="s">
         <v>108</v>
       </c>
-      <c r="F55" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G55" s="93" t="s">
-        <v>204</v>
-      </c>
-      <c r="H55" s="92" t="s">
-        <v>229</v>
-      </c>
-      <c r="I55" s="93" t="s">
-        <v>287</v>
-      </c>
-      <c r="J55" s="92">
+      <c r="F55" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G55" s="92" t="s">
+        <v>195</v>
+      </c>
+      <c r="H55" s="91" t="s">
+        <v>217</v>
+      </c>
+      <c r="I55" s="92" t="s">
+        <v>275</v>
+      </c>
+      <c r="J55" s="91">
         <v>2</v>
       </c>
-      <c r="K55" s="94">
+      <c r="K55" s="93">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L55" s="94"/>
+      <c r="L55" s="93"/>
     </row>
     <row r="56" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="1"/>
@@ -4271,35 +4306,35 @@
         <f t="shared" si="2"/>
         <v>47</v>
       </c>
-      <c r="C56" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D56" s="89" t="s">
+      <c r="C56" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D56" s="88" t="s">
         <v>40</v>
       </c>
-      <c r="E56" s="90" t="s">
+      <c r="E56" s="89" t="s">
         <v>109</v>
       </c>
-      <c r="F56" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G56" s="90" t="s">
-        <v>205</v>
-      </c>
-      <c r="H56" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="I56" s="90" t="s">
-        <v>288</v>
-      </c>
-      <c r="J56" s="89">
+      <c r="F56" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G56" s="89" t="s">
+        <v>196</v>
+      </c>
+      <c r="H56" s="88" t="s">
+        <v>217</v>
+      </c>
+      <c r="I56" s="89" t="s">
+        <v>276</v>
+      </c>
+      <c r="J56" s="88">
         <v>4</v>
       </c>
-      <c r="K56" s="83">
+      <c r="K56" s="82">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L56" s="83"/>
+      <c r="L56" s="82"/>
     </row>
     <row r="57" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="1"/>
@@ -4307,35 +4342,35 @@
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
-      <c r="C57" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D57" s="92" t="s">
+      <c r="C57" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D57" s="91" t="s">
         <v>41</v>
       </c>
-      <c r="E57" s="93" t="s">
+      <c r="E57" s="92" t="s">
         <v>110</v>
       </c>
-      <c r="F57" s="92" t="s">
-        <v>167</v>
-      </c>
-      <c r="G57" s="93" t="s">
-        <v>329</v>
-      </c>
-      <c r="H57" s="92" t="s">
-        <v>250</v>
-      </c>
-      <c r="I57" s="93" t="s">
-        <v>289</v>
-      </c>
-      <c r="J57" s="92">
+      <c r="F57" s="91" t="s">
+        <v>164</v>
+      </c>
+      <c r="G57" s="112" t="s">
+        <v>383</v>
+      </c>
+      <c r="H57" s="91" t="s">
+        <v>238</v>
+      </c>
+      <c r="I57" s="92" t="s">
+        <v>277</v>
+      </c>
+      <c r="J57" s="91">
         <v>4</v>
       </c>
-      <c r="K57" s="94">
+      <c r="K57" s="93">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="L57" s="94"/>
+      <c r="L57" s="93"/>
     </row>
     <row r="58" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="1"/>
@@ -4344,25 +4379,25 @@
         <v>49</v>
       </c>
       <c r="C58" s="60" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D58" s="37" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="E58" s="37" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G58" s="37" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="H58" s="37" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="I58" s="37" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
       <c r="J58" s="37">
         <v>8</v>
@@ -4371,7 +4406,7 @@
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="L58" s="68"/>
+      <c r="L58" s="67"/>
     </row>
     <row r="59" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="1"/>
@@ -4379,35 +4414,35 @@
         <f t="shared" si="2"/>
         <v>50</v>
       </c>
-      <c r="C59" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D59" s="92" t="s">
+      <c r="C59" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D59" s="91" t="s">
         <v>42</v>
       </c>
-      <c r="E59" s="93" t="s">
+      <c r="E59" s="92" t="s">
         <v>112</v>
       </c>
-      <c r="F59" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G59" s="93" t="s">
-        <v>207</v>
-      </c>
-      <c r="H59" s="92" t="s">
-        <v>251</v>
-      </c>
-      <c r="I59" s="93" t="s">
-        <v>291</v>
-      </c>
-      <c r="J59" s="92">
+      <c r="F59" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G59" s="92" t="s">
+        <v>198</v>
+      </c>
+      <c r="H59" s="91" t="s">
+        <v>239</v>
+      </c>
+      <c r="I59" s="92" t="s">
+        <v>279</v>
+      </c>
+      <c r="J59" s="91">
         <v>1</v>
       </c>
-      <c r="K59" s="94">
+      <c r="K59" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L59" s="94"/>
+      <c r="L59" s="93"/>
     </row>
     <row r="60" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="1"/>
@@ -4415,35 +4450,35 @@
         <f t="shared" si="2"/>
         <v>51</v>
       </c>
-      <c r="C60" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D60" s="89" t="s">
+      <c r="C60" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D60" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="E60" s="90" t="s">
+      <c r="E60" s="89" t="s">
         <v>113</v>
       </c>
-      <c r="F60" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G60" s="90" t="s">
-        <v>208</v>
-      </c>
-      <c r="H60" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="I60" s="90" t="s">
-        <v>292</v>
-      </c>
-      <c r="J60" s="89">
+      <c r="F60" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G60" s="89" t="s">
+        <v>199</v>
+      </c>
+      <c r="H60" s="88" t="s">
+        <v>217</v>
+      </c>
+      <c r="I60" s="89" t="s">
+        <v>280</v>
+      </c>
+      <c r="J60" s="88">
         <v>1</v>
       </c>
-      <c r="K60" s="83">
+      <c r="K60" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L60" s="83"/>
+      <c r="L60" s="82"/>
     </row>
     <row r="61" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="1"/>
@@ -4451,35 +4486,35 @@
         <f t="shared" si="2"/>
         <v>52</v>
       </c>
-      <c r="C61" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D61" s="92" t="s">
+      <c r="C61" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D61" s="91" t="s">
         <v>44</v>
       </c>
-      <c r="E61" s="93" t="s">
+      <c r="E61" s="92" t="s">
         <v>114</v>
       </c>
-      <c r="F61" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G61" s="93" t="s">
-        <v>209</v>
-      </c>
-      <c r="H61" s="92" t="s">
-        <v>251</v>
-      </c>
-      <c r="I61" s="93" t="s">
-        <v>293</v>
-      </c>
-      <c r="J61" s="92">
+      <c r="F61" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G61" s="92" t="s">
+        <v>200</v>
+      </c>
+      <c r="H61" s="91" t="s">
+        <v>239</v>
+      </c>
+      <c r="I61" s="92" t="s">
+        <v>281</v>
+      </c>
+      <c r="J61" s="91">
         <v>1</v>
       </c>
-      <c r="K61" s="94">
+      <c r="K61" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L61" s="94"/>
+      <c r="L61" s="93"/>
     </row>
     <row r="62" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="1"/>
@@ -4487,35 +4522,35 @@
         <f t="shared" si="2"/>
         <v>53</v>
       </c>
-      <c r="C62" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D62" s="89" t="s">
+      <c r="C62" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D62" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="E62" s="90" t="s">
+      <c r="E62" s="89" t="s">
         <v>115</v>
       </c>
-      <c r="F62" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G62" s="90" t="s">
-        <v>210</v>
-      </c>
-      <c r="H62" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="I62" s="90" t="s">
-        <v>294</v>
-      </c>
-      <c r="J62" s="89">
+      <c r="F62" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G62" s="89" t="s">
+        <v>201</v>
+      </c>
+      <c r="H62" s="88" t="s">
+        <v>217</v>
+      </c>
+      <c r="I62" s="89" t="s">
+        <v>282</v>
+      </c>
+      <c r="J62" s="88">
         <v>1</v>
       </c>
-      <c r="K62" s="83">
+      <c r="K62" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L62" s="83"/>
+      <c r="L62" s="82"/>
     </row>
     <row r="63" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="1"/>
@@ -4523,35 +4558,35 @@
         <f t="shared" si="2"/>
         <v>54</v>
       </c>
-      <c r="C63" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D63" s="92" t="s">
+      <c r="C63" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D63" s="91" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="93" t="s">
+      <c r="E63" s="92" t="s">
         <v>116</v>
       </c>
-      <c r="F63" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G63" s="93" t="s">
-        <v>211</v>
-      </c>
-      <c r="H63" s="92" t="s">
-        <v>251</v>
-      </c>
-      <c r="I63" s="93" t="s">
-        <v>295</v>
-      </c>
-      <c r="J63" s="92">
+      <c r="F63" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G63" s="92" t="s">
+        <v>202</v>
+      </c>
+      <c r="H63" s="91" t="s">
+        <v>239</v>
+      </c>
+      <c r="I63" s="92" t="s">
+        <v>283</v>
+      </c>
+      <c r="J63" s="91">
         <v>1</v>
       </c>
-      <c r="K63" s="94">
+      <c r="K63" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L63" s="94"/>
+      <c r="L63" s="93"/>
     </row>
     <row r="64" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="1"/>
@@ -4559,35 +4594,35 @@
         <f t="shared" si="2"/>
         <v>55</v>
       </c>
-      <c r="C64" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D64" s="89" t="s">
+      <c r="C64" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D64" s="88" t="s">
         <v>47</v>
       </c>
-      <c r="E64" s="90" t="s">
+      <c r="E64" s="89" t="s">
         <v>117</v>
       </c>
-      <c r="F64" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G64" s="90" t="s">
-        <v>212</v>
-      </c>
-      <c r="H64" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="I64" s="90" t="s">
-        <v>296</v>
-      </c>
-      <c r="J64" s="89">
+      <c r="F64" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G64" s="89" t="s">
+        <v>203</v>
+      </c>
+      <c r="H64" s="88" t="s">
+        <v>217</v>
+      </c>
+      <c r="I64" s="89" t="s">
+        <v>284</v>
+      </c>
+      <c r="J64" s="88">
         <v>1</v>
       </c>
-      <c r="K64" s="83">
+      <c r="K64" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L64" s="83"/>
+      <c r="L64" s="82"/>
     </row>
     <row r="65" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="1"/>
@@ -4595,35 +4630,35 @@
         <f t="shared" si="2"/>
         <v>56</v>
       </c>
-      <c r="C65" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D65" s="92" t="s">
+      <c r="C65" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D65" s="91" t="s">
         <v>48</v>
       </c>
-      <c r="E65" s="93" t="s">
+      <c r="E65" s="92" t="s">
         <v>118</v>
       </c>
-      <c r="F65" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G65" s="93" t="s">
-        <v>213</v>
-      </c>
-      <c r="H65" s="92" t="s">
-        <v>229</v>
-      </c>
-      <c r="I65" s="93" t="s">
-        <v>297</v>
-      </c>
-      <c r="J65" s="92">
+      <c r="F65" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G65" s="92" t="s">
+        <v>204</v>
+      </c>
+      <c r="H65" s="91" t="s">
+        <v>217</v>
+      </c>
+      <c r="I65" s="92" t="s">
+        <v>285</v>
+      </c>
+      <c r="J65" s="91">
         <v>1</v>
       </c>
-      <c r="K65" s="94">
+      <c r="K65" s="93">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L65" s="94"/>
+      <c r="L65" s="93"/>
     </row>
     <row r="66" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="1"/>
@@ -4631,35 +4666,35 @@
         <f t="shared" si="2"/>
         <v>57</v>
       </c>
-      <c r="C66" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D66" s="89" t="s">
+      <c r="C66" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D66" s="88" t="s">
         <v>49</v>
       </c>
-      <c r="E66" s="90" t="s">
+      <c r="E66" s="89" t="s">
         <v>119</v>
       </c>
-      <c r="F66" s="89" t="s">
-        <v>166</v>
-      </c>
-      <c r="G66" s="90" t="s">
-        <v>214</v>
-      </c>
-      <c r="H66" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="I66" s="90" t="s">
-        <v>298</v>
-      </c>
-      <c r="J66" s="89">
+      <c r="F66" s="88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G66" s="113" t="s">
+        <v>384</v>
+      </c>
+      <c r="H66" s="88" t="s">
+        <v>217</v>
+      </c>
+      <c r="I66" s="89" t="s">
+        <v>286</v>
+      </c>
+      <c r="J66" s="88">
         <v>1</v>
       </c>
-      <c r="K66" s="83">
+      <c r="K66" s="82">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L66" s="83"/>
+      <c r="L66" s="82"/>
     </row>
     <row r="67" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="1"/>
@@ -4667,35 +4702,35 @@
         <f t="shared" si="2"/>
         <v>58</v>
       </c>
-      <c r="C67" s="91" t="s">
-        <v>324</v>
-      </c>
-      <c r="D67" s="92" t="s">
-        <v>372</v>
-      </c>
-      <c r="E67" s="93" t="s">
+      <c r="C67" s="90" t="s">
+        <v>312</v>
+      </c>
+      <c r="D67" s="91" t="s">
+        <v>359</v>
+      </c>
+      <c r="E67" s="92" t="s">
         <v>120</v>
       </c>
-      <c r="F67" s="92" t="s">
-        <v>166</v>
-      </c>
-      <c r="G67" s="93" t="s">
-        <v>215</v>
-      </c>
-      <c r="H67" s="92" t="s">
-        <v>229</v>
-      </c>
-      <c r="I67" s="93" t="s">
-        <v>299</v>
-      </c>
-      <c r="J67" s="92">
+      <c r="F67" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="G67" s="92" t="s">
+        <v>205</v>
+      </c>
+      <c r="H67" s="91" t="s">
+        <v>217</v>
+      </c>
+      <c r="I67" s="92" t="s">
+        <v>287</v>
+      </c>
+      <c r="J67" s="91">
         <v>2</v>
       </c>
-      <c r="K67" s="94">
+      <c r="K67" s="93">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L67" s="94"/>
+      <c r="L67" s="93"/>
     </row>
     <row r="68" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="1"/>
@@ -4704,7 +4739,7 @@
         <v>59</v>
       </c>
       <c r="C68" s="60" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D68" s="37" t="s">
         <v>50</v>
@@ -4713,16 +4748,16 @@
         <v>121</v>
       </c>
       <c r="F68" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="H68" s="37" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I68" s="38" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="J68" s="37">
         <v>2</v>
@@ -4740,25 +4775,25 @@
         <v>60</v>
       </c>
       <c r="C69" s="59" t="s">
-        <v>324</v>
-      </c>
-      <c r="D69" s="77" t="s">
-        <v>339</v>
+        <v>312</v>
+      </c>
+      <c r="D69" s="76" t="s">
+        <v>326</v>
       </c>
       <c r="E69" s="40" t="s">
         <v>111</v>
       </c>
       <c r="F69" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G69" s="40" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="H69" s="39" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I69" s="40" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="J69" s="39">
         <v>1</v>
@@ -4767,7 +4802,7 @@
         <f>J69*20</f>
         <v>20</v>
       </c>
-      <c r="L69" s="69"/>
+      <c r="L69" s="68"/>
     </row>
     <row r="70" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="1"/>
@@ -4776,7 +4811,7 @@
         <v>61</v>
       </c>
       <c r="C70" s="60" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D70" s="37" t="s">
         <v>51</v>
@@ -4785,16 +4820,16 @@
         <v>122</v>
       </c>
       <c r="F70" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G70" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="H70" s="37" t="s">
         <v>217</v>
       </c>
-      <c r="H70" s="37" t="s">
-        <v>229</v>
-      </c>
       <c r="I70" s="38" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="J70" s="37">
         <v>2</v>
@@ -4812,7 +4847,7 @@
         <v>62</v>
       </c>
       <c r="C71" s="59" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D71" s="39" t="s">
         <v>52</v>
@@ -4821,16 +4856,16 @@
         <v>123</v>
       </c>
       <c r="F71" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G71" s="40" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="H71" s="39" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="I71" s="40" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="J71" s="39">
         <v>1</v>
@@ -4848,25 +4883,25 @@
         <v>63</v>
       </c>
       <c r="C72" s="60" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D72" s="37" t="s">
         <v>53</v>
       </c>
       <c r="E72" s="38" t="s">
+        <v>333</v>
+      </c>
+      <c r="F72" s="75" t="s">
+        <v>163</v>
+      </c>
+      <c r="G72" s="38" t="s">
+        <v>347</v>
+      </c>
+      <c r="H72" s="37" t="s">
+        <v>240</v>
+      </c>
+      <c r="I72" s="38" t="s">
         <v>346</v>
-      </c>
-      <c r="F72" s="76" t="s">
-        <v>166</v>
-      </c>
-      <c r="G72" s="38" t="s">
-        <v>360</v>
-      </c>
-      <c r="H72" s="37" t="s">
-        <v>252</v>
-      </c>
-      <c r="I72" s="38" t="s">
-        <v>359</v>
       </c>
       <c r="J72" s="37">
         <v>1</v>
@@ -4875,7 +4910,7 @@
         <f t="shared" ref="K72:K90" si="3">J72*20</f>
         <v>20</v>
       </c>
-      <c r="L72" s="68"/>
+      <c r="L72" s="67"/>
     </row>
     <row r="73" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="1"/>
@@ -4884,25 +4919,25 @@
         <v>64</v>
       </c>
       <c r="C73" s="59" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D73" s="39" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
       <c r="E73" s="40" t="s">
         <v>127</v>
       </c>
       <c r="F73" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G73" s="40" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="H73" s="39" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I73" s="40" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="J73" s="39">
         <v>6</v>
@@ -4911,7 +4946,7 @@
         <f>J73*20</f>
         <v>120</v>
       </c>
-      <c r="L73" s="69"/>
+      <c r="L73" s="68"/>
     </row>
     <row r="74" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="1"/>
@@ -4920,7 +4955,7 @@
         <v>65</v>
       </c>
       <c r="C74" s="60" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D74" s="37" t="s">
         <v>54</v>
@@ -4929,16 +4964,16 @@
         <v>124</v>
       </c>
       <c r="F74" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G74" s="38" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
       <c r="H74" s="37" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="I74" s="38" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="J74" s="37">
         <v>1</v>
@@ -4956,7 +4991,7 @@
         <v>66</v>
       </c>
       <c r="C75" s="59" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="D75" s="39" t="s">
         <v>55</v>
@@ -4965,16 +5000,16 @@
         <v>125</v>
       </c>
       <c r="F75" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G75" s="40" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="H75" s="39" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="I75" s="40" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="J75" s="39">
         <v>1</v>
@@ -4991,36 +5026,36 @@
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
-      <c r="C76" s="84" t="s">
-        <v>324</v>
-      </c>
-      <c r="D76" s="85" t="s">
+      <c r="C76" s="83" t="s">
+        <v>312</v>
+      </c>
+      <c r="D76" s="84" t="s">
         <v>56</v>
       </c>
-      <c r="E76" s="86" t="s">
+      <c r="E76" s="85" t="s">
         <v>126</v>
       </c>
-      <c r="F76" s="85" t="s">
-        <v>168</v>
-      </c>
-      <c r="G76" s="86" t="s">
-        <v>219</v>
-      </c>
-      <c r="H76" s="85" t="s">
-        <v>229</v>
-      </c>
-      <c r="I76" s="86" t="s">
-        <v>305</v>
-      </c>
-      <c r="J76" s="85">
+      <c r="F76" s="84" t="s">
+        <v>165</v>
+      </c>
+      <c r="G76" s="85" t="s">
+        <v>209</v>
+      </c>
+      <c r="H76" s="84" t="s">
+        <v>217</v>
+      </c>
+      <c r="I76" s="85" t="s">
+        <v>293</v>
+      </c>
+      <c r="J76" s="84">
         <v>4</v>
       </c>
-      <c r="K76" s="63">
+      <c r="K76" s="62">
         <f t="shared" si="3"/>
         <v>80</v>
       </c>
-      <c r="L76" s="63" t="s">
-        <v>362</v>
+      <c r="L76" s="62" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -5029,36 +5064,36 @@
         <f t="shared" si="2"/>
         <v>68</v>
       </c>
-      <c r="C77" s="84" t="s">
-        <v>169</v>
-      </c>
-      <c r="D77" s="85" t="s">
-        <v>363</v>
-      </c>
-      <c r="E77" s="86" t="s">
+      <c r="C77" s="83" t="s">
+        <v>166</v>
+      </c>
+      <c r="D77" s="84" t="s">
+        <v>350</v>
+      </c>
+      <c r="E77" s="85" t="s">
         <v>128</v>
       </c>
-      <c r="F77" s="85" t="s">
-        <v>169</v>
-      </c>
-      <c r="G77" s="86" t="s">
-        <v>314</v>
-      </c>
-      <c r="H77" s="85" t="s">
-        <v>314</v>
-      </c>
-      <c r="I77" s="86" t="s">
-        <v>314</v>
-      </c>
-      <c r="J77" s="85">
+      <c r="F77" s="84" t="s">
+        <v>166</v>
+      </c>
+      <c r="G77" s="85" t="s">
+        <v>302</v>
+      </c>
+      <c r="H77" s="84" t="s">
+        <v>302</v>
+      </c>
+      <c r="I77" s="85" t="s">
+        <v>302</v>
+      </c>
+      <c r="J77" s="84">
         <v>15</v>
       </c>
-      <c r="K77" s="63">
+      <c r="K77" s="62">
         <f t="shared" si="3"/>
         <v>300</v>
       </c>
-      <c r="L77" s="63" t="s">
-        <v>337</v>
+      <c r="L77" s="62" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -5067,35 +5102,35 @@
         <f t="shared" si="2"/>
         <v>69</v>
       </c>
-      <c r="C78" s="88" t="s">
-        <v>326</v>
-      </c>
-      <c r="D78" s="89" t="s">
+      <c r="C78" s="87" t="s">
+        <v>314</v>
+      </c>
+      <c r="D78" s="88" t="s">
         <v>57</v>
       </c>
-      <c r="E78" s="90" t="s">
+      <c r="E78" s="89" t="s">
         <v>129</v>
       </c>
-      <c r="F78" s="89" t="s">
-        <v>170</v>
-      </c>
-      <c r="G78" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="H78" s="89" t="s">
-        <v>254</v>
-      </c>
-      <c r="I78" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J78" s="89">
+      <c r="F78" s="88" t="s">
+        <v>167</v>
+      </c>
+      <c r="G78" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="H78" s="88" t="s">
+        <v>242</v>
+      </c>
+      <c r="I78" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J78" s="88">
         <v>1</v>
       </c>
-      <c r="K78" s="83">
+      <c r="K78" s="82">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L78" s="83"/>
+      <c r="L78" s="82"/>
     </row>
     <row r="79" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="1"/>
@@ -5103,35 +5138,35 @@
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
-      <c r="C79" s="91" t="s">
-        <v>327</v>
-      </c>
-      <c r="D79" s="92" t="s">
+      <c r="C79" s="90" t="s">
+        <v>315</v>
+      </c>
+      <c r="D79" s="91" t="s">
         <v>58</v>
       </c>
-      <c r="E79" s="93" t="s">
+      <c r="E79" s="92" t="s">
         <v>130</v>
       </c>
-      <c r="F79" s="92" t="s">
-        <v>308</v>
-      </c>
-      <c r="G79" s="93">
+      <c r="F79" s="91" t="s">
+        <v>296</v>
+      </c>
+      <c r="G79" s="92">
         <v>750314597</v>
       </c>
-      <c r="H79" s="92" t="s">
-        <v>255</v>
-      </c>
-      <c r="I79" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J79" s="92">
+      <c r="H79" s="91" t="s">
+        <v>243</v>
+      </c>
+      <c r="I79" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J79" s="91">
         <v>1</v>
       </c>
-      <c r="K79" s="94">
+      <c r="K79" s="93">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L79" s="94"/>
+      <c r="L79" s="93"/>
     </row>
     <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="1"/>
@@ -5139,35 +5174,35 @@
         <f t="shared" si="2"/>
         <v>71</v>
       </c>
-      <c r="C80" s="88" t="s">
-        <v>328</v>
-      </c>
-      <c r="D80" s="89" t="s">
+      <c r="C80" s="87" t="s">
+        <v>316</v>
+      </c>
+      <c r="D80" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="E80" s="90" t="s">
+      <c r="E80" s="89" t="s">
         <v>131</v>
       </c>
-      <c r="F80" s="89" t="s">
-        <v>308</v>
-      </c>
-      <c r="G80" s="90" t="s">
-        <v>171</v>
-      </c>
-      <c r="H80" s="89" t="s">
-        <v>256</v>
-      </c>
-      <c r="I80" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J80" s="89">
+      <c r="F80" s="88" t="s">
+        <v>296</v>
+      </c>
+      <c r="G80" s="89" t="s">
+        <v>168</v>
+      </c>
+      <c r="H80" s="88" t="s">
+        <v>244</v>
+      </c>
+      <c r="I80" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J80" s="88">
         <v>1</v>
       </c>
-      <c r="K80" s="83">
+      <c r="K80" s="82">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L80" s="83"/>
+      <c r="L80" s="82"/>
     </row>
     <row r="81" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
@@ -5175,35 +5210,35 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="C81" s="91" t="s">
-        <v>328</v>
-      </c>
-      <c r="D81" s="92" t="s">
+      <c r="C81" s="90" t="s">
+        <v>316</v>
+      </c>
+      <c r="D81" s="91" t="s">
         <v>60</v>
       </c>
-      <c r="E81" s="93" t="s">
+      <c r="E81" s="92" t="s">
         <v>132</v>
       </c>
-      <c r="F81" s="92" t="s">
-        <v>172</v>
-      </c>
-      <c r="G81" s="93" t="s">
-        <v>221</v>
-      </c>
-      <c r="H81" s="92" t="s">
-        <v>257</v>
-      </c>
-      <c r="I81" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J81" s="92">
+      <c r="F81" s="91" t="s">
+        <v>169</v>
+      </c>
+      <c r="G81" s="114" t="s">
+        <v>385</v>
+      </c>
+      <c r="H81" s="91" t="s">
+        <v>245</v>
+      </c>
+      <c r="I81" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J81" s="91">
         <v>1</v>
       </c>
-      <c r="K81" s="94">
+      <c r="K81" s="93">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L81" s="71"/>
+      <c r="L81" s="70"/>
     </row>
     <row r="82" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="1"/>
@@ -5211,35 +5246,35 @@
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
-      <c r="C82" s="88" t="s">
-        <v>328</v>
-      </c>
-      <c r="D82" s="89" t="s">
+      <c r="C82" s="87" t="s">
+        <v>316</v>
+      </c>
+      <c r="D82" s="88" t="s">
         <v>61</v>
       </c>
-      <c r="E82" s="90" t="s">
+      <c r="E82" s="89" t="s">
         <v>133</v>
       </c>
-      <c r="F82" s="89" t="s">
-        <v>173</v>
-      </c>
-      <c r="G82" s="90" t="s">
-        <v>222</v>
-      </c>
-      <c r="H82" s="89" t="s">
-        <v>256</v>
-      </c>
-      <c r="I82" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J82" s="89">
+      <c r="F82" s="88" t="s">
+        <v>170</v>
+      </c>
+      <c r="G82" s="115" t="s">
+        <v>386</v>
+      </c>
+      <c r="H82" s="88" t="s">
+        <v>244</v>
+      </c>
+      <c r="I82" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J82" s="88">
         <v>1</v>
       </c>
-      <c r="K82" s="83">
+      <c r="K82" s="82">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L82" s="70"/>
+      <c r="L82" s="69"/>
     </row>
     <row r="83" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="1"/>
@@ -5247,35 +5282,35 @@
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
-      <c r="C83" s="91" t="s">
-        <v>328</v>
-      </c>
-      <c r="D83" s="92" t="s">
+      <c r="C83" s="90" t="s">
+        <v>316</v>
+      </c>
+      <c r="D83" s="91" t="s">
         <v>62</v>
       </c>
-      <c r="E83" s="93" t="s">
+      <c r="E83" s="92" t="s">
         <v>134</v>
       </c>
-      <c r="F83" s="92" t="s">
-        <v>310</v>
-      </c>
-      <c r="G83" s="93" t="s">
-        <v>174</v>
-      </c>
-      <c r="H83" s="92" t="s">
-        <v>256</v>
-      </c>
-      <c r="I83" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J83" s="92">
+      <c r="F83" s="91" t="s">
+        <v>298</v>
+      </c>
+      <c r="G83" s="92" t="s">
+        <v>171</v>
+      </c>
+      <c r="H83" s="91" t="s">
+        <v>244</v>
+      </c>
+      <c r="I83" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J83" s="91">
         <v>1</v>
       </c>
-      <c r="K83" s="94">
+      <c r="K83" s="93">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L83" s="94"/>
+      <c r="L83" s="93"/>
     </row>
     <row r="84" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="1"/>
@@ -5283,35 +5318,35 @@
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
-      <c r="C84" s="88" t="s">
-        <v>328</v>
-      </c>
-      <c r="D84" s="89" t="s">
+      <c r="C84" s="87" t="s">
+        <v>316</v>
+      </c>
+      <c r="D84" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="E84" s="90" t="s">
+      <c r="E84" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="F84" s="89" t="s">
-        <v>175</v>
-      </c>
-      <c r="G84" s="90" t="s">
-        <v>223</v>
-      </c>
-      <c r="H84" s="89" t="s">
-        <v>256</v>
-      </c>
-      <c r="I84" s="90" t="s">
-        <v>314</v>
-      </c>
-      <c r="J84" s="89">
+      <c r="F84" s="88" t="s">
+        <v>172</v>
+      </c>
+      <c r="G84" s="89" t="s">
+        <v>211</v>
+      </c>
+      <c r="H84" s="88" t="s">
+        <v>244</v>
+      </c>
+      <c r="I84" s="89" t="s">
+        <v>302</v>
+      </c>
+      <c r="J84" s="88">
         <v>1</v>
       </c>
-      <c r="K84" s="83">
+      <c r="K84" s="82">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L84" s="83"/>
+      <c r="L84" s="82"/>
     </row>
     <row r="85" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="1"/>
@@ -5319,38 +5354,38 @@
         <f t="shared" si="2"/>
         <v>76</v>
       </c>
-      <c r="C85" s="64" t="s">
-        <v>328</v>
-      </c>
-      <c r="D85" s="65" t="s">
+      <c r="C85" s="63" t="s">
+        <v>316</v>
+      </c>
+      <c r="D85" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="E85" s="66" t="s">
+      <c r="E85" s="65" t="s">
         <v>136</v>
       </c>
-      <c r="F85" s="65" t="s">
-        <v>176</v>
-      </c>
-      <c r="G85" s="66" t="s">
-        <v>224</v>
-      </c>
-      <c r="H85" s="65" t="s">
-        <v>258</v>
-      </c>
-      <c r="I85" s="66" t="s">
-        <v>314</v>
-      </c>
-      <c r="J85" s="65">
+      <c r="F85" s="64" t="s">
+        <v>173</v>
+      </c>
+      <c r="G85" s="65" t="s">
+        <v>212</v>
+      </c>
+      <c r="H85" s="64" t="s">
+        <v>246</v>
+      </c>
+      <c r="I85" s="65" t="s">
+        <v>302</v>
+      </c>
+      <c r="J85" s="64">
         <v>1</v>
       </c>
-      <c r="K85" s="67">
+      <c r="K85" s="66">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L85" s="67" t="s">
-        <v>348</v>
-      </c>
-      <c r="O85" s="99"/>
+      <c r="L85" s="66" t="s">
+        <v>335</v>
+      </c>
+      <c r="O85" s="98"/>
     </row>
     <row r="86" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="1"/>
@@ -5358,35 +5393,35 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="C86" s="88" t="s">
-        <v>328</v>
-      </c>
-      <c r="D86" s="89" t="s">
+      <c r="C86" s="87" t="s">
+        <v>316</v>
+      </c>
+      <c r="D86" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="E86" s="90" t="s">
+      <c r="E86" s="89" t="s">
         <v>137</v>
       </c>
-      <c r="F86" s="89" t="s">
-        <v>177</v>
-      </c>
-      <c r="G86" s="90" t="s">
-        <v>225</v>
-      </c>
-      <c r="H86" s="89" t="s">
-        <v>259</v>
-      </c>
-      <c r="I86" s="97" t="s">
-        <v>314</v>
-      </c>
-      <c r="J86" s="89">
+      <c r="F86" s="88" t="s">
+        <v>174</v>
+      </c>
+      <c r="G86" s="89" t="s">
+        <v>213</v>
+      </c>
+      <c r="H86" s="88" t="s">
+        <v>247</v>
+      </c>
+      <c r="I86" s="96" t="s">
+        <v>302</v>
+      </c>
+      <c r="J86" s="88">
         <v>1</v>
       </c>
-      <c r="K86" s="83">
+      <c r="K86" s="82">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L86" s="83"/>
+      <c r="L86" s="82"/>
     </row>
     <row r="87" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="1"/>
@@ -5394,35 +5429,35 @@
         <f t="shared" si="2"/>
         <v>78</v>
       </c>
-      <c r="C87" s="91" t="s">
-        <v>328</v>
-      </c>
-      <c r="D87" s="92" t="s">
-        <v>364</v>
-      </c>
-      <c r="E87" s="93" t="s">
+      <c r="C87" s="90" t="s">
+        <v>316</v>
+      </c>
+      <c r="D87" s="91" t="s">
+        <v>351</v>
+      </c>
+      <c r="E87" s="92" t="s">
         <v>138</v>
       </c>
-      <c r="F87" s="92" t="s">
-        <v>311</v>
-      </c>
-      <c r="G87" s="93" t="s">
-        <v>178</v>
-      </c>
-      <c r="H87" s="92" t="s">
-        <v>256</v>
-      </c>
-      <c r="I87" s="93" t="s">
-        <v>314</v>
-      </c>
-      <c r="J87" s="98">
+      <c r="F87" s="91" t="s">
+        <v>299</v>
+      </c>
+      <c r="G87" s="116" t="s">
+        <v>387</v>
+      </c>
+      <c r="H87" s="91" t="s">
+        <v>244</v>
+      </c>
+      <c r="I87" s="92" t="s">
+        <v>302</v>
+      </c>
+      <c r="J87" s="97">
         <v>2</v>
       </c>
-      <c r="K87" s="94">
+      <c r="K87" s="93">
         <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="L87" s="71"/>
+      <c r="L87" s="70"/>
     </row>
     <row r="88" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="1"/>
@@ -5431,7 +5466,7 @@
         <v>79</v>
       </c>
       <c r="C88" s="60" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="D88" s="37" t="s">
         <v>66</v>
@@ -5440,16 +5475,16 @@
         <v>140</v>
       </c>
       <c r="F88" s="37" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="G88" s="38" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="H88" s="37" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="I88" s="38" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="J88" s="37">
         <v>1</v>
@@ -5467,25 +5502,25 @@
         <v>80</v>
       </c>
       <c r="C89" s="59" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="D89" s="39" t="s">
-        <v>365</v>
+        <v>352</v>
       </c>
       <c r="E89" s="40" t="s">
         <v>139</v>
       </c>
       <c r="F89" s="39" t="s">
-        <v>312</v>
-      </c>
-      <c r="G89" s="40" t="s">
-        <v>179</v>
+        <v>300</v>
+      </c>
+      <c r="G89" s="117" t="s">
+        <v>388</v>
       </c>
       <c r="H89" s="39" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="I89" s="40" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="J89" s="39">
         <v>1</v>
@@ -5494,7 +5529,7 @@
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L89" s="71"/>
+      <c r="L89" s="70"/>
     </row>
     <row r="90" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="1"/>
@@ -5503,22 +5538,22 @@
         <v>81</v>
       </c>
       <c r="C90" s="59" t="s">
-        <v>380</v>
+        <v>367</v>
       </c>
       <c r="D90" s="39" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="E90" s="40" t="s">
-        <v>383</v>
+        <v>370</v>
       </c>
       <c r="F90" s="39" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="G90" s="40" t="s">
-        <v>381</v>
+        <v>368</v>
       </c>
       <c r="H90" s="39" t="s">
-        <v>382</v>
+        <v>369</v>
       </c>
       <c r="I90" s="40"/>
       <c r="J90" s="39">
@@ -5528,7 +5563,7 @@
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L90" s="71"/>
+      <c r="L90" s="70"/>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A91" s="1"/>

</xml_diff>

<commit_message>
#152 C1 Alternate Part No Updated in BOMs.
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/Supplier BOM_Top (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/Supplier BOM_Top (20 Boards).xlsx
@@ -1,20 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25726"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBA2E67-D6F2-4229-B541-2CDCE80DA94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -445,9 +456,6 @@
   </si>
   <si>
     <t>Footprint</t>
-  </si>
-  <si>
-    <t>UCD1H221MNL1GS</t>
   </si>
   <si>
     <t>Cap 0603</t>
@@ -1321,11 +1329,14 @@
   <si>
     <t>ISO6761FDWR</t>
   </si>
+  <si>
+    <t>EEEFT1H221AP</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1787,22 +1798,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1812,18 +1823,18 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1838,7 +1849,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1848,8 +1859,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1861,22 +1872,22 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1898,31 +1909,31 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1932,7 +1943,7 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1950,7 +1961,7 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2059,10 +2070,10 @@
     <xf numFmtId="0" fontId="23" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2073,51 +2084,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2458,25 +2424,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O92"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.1796875" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.7265625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="30.1796875" customWidth="1"/>
-    <col min="7" max="7" width="33.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.453125" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2490,7 +2456,7 @@
       <c r="K1" s="100"/>
       <c r="L1" s="100"/>
     </row>
-    <row r="2" spans="1:12" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -2499,7 +2465,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="54" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -2508,7 +2474,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="43"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -2517,7 +2483,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="55" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -2526,7 +2492,7 @@
       <c r="K3" s="4"/>
       <c r="L3" s="101"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -2535,7 +2501,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="56" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -2544,7 +2510,7 @@
       <c r="K4" s="61"/>
       <c r="L4" s="102"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -2560,7 +2526,7 @@
       <c r="K5" s="61"/>
       <c r="L5" s="102"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -2574,7 +2540,7 @@
       <c r="K6" s="61"/>
       <c r="L6" s="102"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -2588,7 +2554,7 @@
       <c r="K7" s="7"/>
       <c r="L7" s="102"/>
     </row>
-    <row r="8" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -2602,13 +2568,13 @@
       <c r="K8" s="7"/>
       <c r="L8" s="102"/>
     </row>
-    <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>7</v>
@@ -2620,32 +2586,32 @@
         <v>141</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="K9" s="31" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L9" s="31" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>8</v>
@@ -2654,16 +2620,16 @@
         <v>68</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>142</v>
+        <v>388</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J10" s="37">
         <v>1</v>
@@ -2674,32 +2640,32 @@
       </c>
       <c r="L10" s="41"/>
     </row>
-    <row r="11" spans="1:12" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
         <f t="shared" ref="B11:B45" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="71" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D11" s="72" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E11" s="73" t="s">
         <v>69</v>
       </c>
       <c r="F11" s="72" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G11" s="73" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H11" s="72" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I11" s="73" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J11" s="72">
         <v>15</v>
@@ -2709,35 +2675,35 @@
         <v>300</v>
       </c>
       <c r="L11" s="74" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E12" s="38" t="s">
         <v>70</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J12" s="75">
         <v>2</v>
@@ -2748,32 +2714,32 @@
       </c>
       <c r="L12" s="67"/>
     </row>
-    <row r="13" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D13" s="39" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E13" s="40" t="s">
         <v>71</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I13" s="40" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J13" s="76">
         <v>1</v>
@@ -2784,32 +2750,32 @@
       </c>
       <c r="L13" s="68"/>
     </row>
-    <row r="14" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
       <c r="C14" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E14" s="38" t="s">
         <v>72</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J14" s="37">
         <v>8</v>
@@ -2820,32 +2786,32 @@
       </c>
       <c r="L14" s="67"/>
     </row>
-    <row r="15" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D15" s="39" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E15" s="40" t="s">
         <v>73</v>
       </c>
       <c r="F15" s="39" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I15" s="40" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J15" s="76">
         <v>3</v>
@@ -2856,32 +2822,32 @@
       </c>
       <c r="L15" s="68"/>
     </row>
-    <row r="16" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
       <c r="C16" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G16" s="86" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H16" s="75" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J16" s="37">
         <v>6</v>
@@ -2892,14 +2858,14 @@
       </c>
       <c r="L16" s="67"/>
     </row>
-    <row r="17" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C17" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>9</v>
@@ -2908,16 +2874,16 @@
         <v>74</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I17" s="40" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J17" s="39">
         <v>1</v>
@@ -2928,32 +2894,32 @@
       </c>
       <c r="L17" s="42"/>
     </row>
-    <row r="18" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="87" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D18" s="88" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E18" s="89" t="s">
         <v>75</v>
       </c>
       <c r="F18" s="88" t="s">
-        <v>145</v>
-      </c>
-      <c r="G18" s="103" t="s">
-        <v>375</v>
+        <v>144</v>
+      </c>
+      <c r="G18" s="88" t="s">
+        <v>374</v>
       </c>
       <c r="H18" s="88" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I18" s="89" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J18" s="88">
         <v>8</v>
@@ -2964,14 +2930,14 @@
       </c>
       <c r="L18" s="82"/>
     </row>
-    <row r="19" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
       <c r="C19" s="90" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D19" s="91" t="s">
         <v>10</v>
@@ -2980,16 +2946,16 @@
         <v>76</v>
       </c>
       <c r="F19" s="91" t="s">
-        <v>143</v>
-      </c>
-      <c r="G19" s="104" t="s">
-        <v>376</v>
+        <v>142</v>
+      </c>
+      <c r="G19" s="91" t="s">
+        <v>375</v>
       </c>
       <c r="H19" s="91" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I19" s="92" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J19" s="91">
         <v>1</v>
@@ -3000,14 +2966,14 @@
       </c>
       <c r="L19" s="93"/>
     </row>
-    <row r="20" spans="1:12" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="87" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D20" s="88" t="s">
         <v>11</v>
@@ -3016,16 +2982,16 @@
         <v>77</v>
       </c>
       <c r="F20" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G20" s="88" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H20" s="88" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I20" s="89" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J20" s="88">
         <v>1</v>
@@ -3036,14 +3002,14 @@
       </c>
       <c r="L20" s="82"/>
     </row>
-    <row r="21" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
       <c r="C21" s="90" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D21" s="91" t="s">
         <v>12</v>
@@ -3052,16 +3018,16 @@
         <v>78</v>
       </c>
       <c r="F21" s="91" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G21" s="92" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H21" s="91" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I21" s="92" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J21" s="91">
         <v>2</v>
@@ -3072,14 +3038,14 @@
       </c>
       <c r="L21" s="93"/>
     </row>
-    <row r="22" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
       <c r="C22" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D22" s="37" t="s">
         <v>13</v>
@@ -3088,16 +3054,16 @@
         <v>79</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J22" s="37">
         <v>1</v>
@@ -3108,32 +3074,32 @@
       </c>
       <c r="L22" s="41"/>
     </row>
-    <row r="23" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D23" s="39" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E23" s="40" t="s">
         <v>80</v>
       </c>
       <c r="F23" s="39" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G23" s="40" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H23" s="39" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I23" s="40" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J23" s="39">
         <v>1</v>
@@ -3144,14 +3110,14 @@
       </c>
       <c r="L23" s="68"/>
     </row>
-    <row r="24" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
       <c r="C24" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D24" s="37" t="s">
         <v>14</v>
@@ -3160,16 +3126,16 @@
         <v>81</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="G24" s="105" t="s">
-        <v>377</v>
+        <v>143</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>376</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J24" s="37">
         <v>1</v>
@@ -3180,14 +3146,14 @@
       </c>
       <c r="L24" s="41"/>
     </row>
-    <row r="25" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D25" s="39" t="s">
         <v>15</v>
@@ -3196,16 +3162,16 @@
         <v>82</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G25" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J25" s="39">
         <v>1</v>
@@ -3216,32 +3182,32 @@
       </c>
       <c r="L25" s="42"/>
     </row>
-    <row r="26" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="87" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D26" s="88" t="s">
         <v>16</v>
       </c>
       <c r="E26" s="94" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F26" s="88" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G26" s="94" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H26" s="95" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I26" s="94" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J26" s="88">
         <v>1</v>
@@ -3252,32 +3218,32 @@
       </c>
       <c r="L26" s="67"/>
     </row>
-    <row r="27" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
       <c r="C27" s="90" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D27" s="91" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E27" s="92" t="s">
         <v>83</v>
       </c>
       <c r="F27" s="91" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G27" s="92" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H27" s="91" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="I27" s="92" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J27" s="91">
         <v>1</v>
@@ -3288,14 +3254,14 @@
       </c>
       <c r="L27" s="70"/>
     </row>
-    <row r="28" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D28" s="37" t="s">
         <v>17</v>
@@ -3304,16 +3270,16 @@
         <v>84</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J28" s="37">
         <v>1</v>
@@ -3324,14 +3290,14 @@
       </c>
       <c r="L28" s="41"/>
     </row>
-    <row r="29" spans="1:12" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C29" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D29" s="39" t="s">
         <v>18</v>
@@ -3340,16 +3306,16 @@
         <v>85</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J29" s="39">
         <v>1</v>
@@ -3360,14 +3326,14 @@
       </c>
       <c r="L29" s="42"/>
     </row>
-    <row r="30" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="60" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D30" s="37" t="s">
         <v>19</v>
@@ -3376,16 +3342,16 @@
         <v>86</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H30" s="37" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I30" s="38" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J30" s="37">
         <v>1</v>
@@ -3396,14 +3362,14 @@
       </c>
       <c r="L30" s="41"/>
     </row>
-    <row r="31" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D31" s="91" t="s">
         <v>20</v>
@@ -3412,16 +3378,16 @@
         <v>87</v>
       </c>
       <c r="F31" s="91" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G31" s="92" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H31" s="91" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I31" s="92" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J31" s="91">
         <v>4</v>
@@ -3432,14 +3398,14 @@
       </c>
       <c r="L31" s="93"/>
     </row>
-    <row r="32" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C32" s="87" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D32" s="88" t="s">
         <v>21</v>
@@ -3448,16 +3414,16 @@
         <v>88</v>
       </c>
       <c r="F32" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G32" s="89" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H32" s="88" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I32" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J32" s="88">
         <v>1</v>
@@ -3468,14 +3434,14 @@
       </c>
       <c r="L32" s="82"/>
     </row>
-    <row r="33" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
       <c r="C33" s="90" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D33" s="91" t="s">
         <v>22</v>
@@ -3484,16 +3450,16 @@
         <v>89</v>
       </c>
       <c r="F33" s="91" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G33" s="92" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H33" s="91" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I33" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J33" s="91">
         <v>1</v>
@@ -3504,32 +3470,32 @@
       </c>
       <c r="L33" s="93"/>
     </row>
-    <row r="34" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C34" s="87" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D34" s="88" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E34" s="89" t="s">
         <v>90</v>
       </c>
       <c r="F34" s="88" t="s">
-        <v>151</v>
-      </c>
-      <c r="G34" s="106" t="s">
-        <v>269</v>
+        <v>150</v>
+      </c>
+      <c r="G34" s="88" t="s">
+        <v>268</v>
       </c>
       <c r="H34" s="88" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I34" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J34" s="88">
         <v>2</v>
@@ -3540,32 +3506,32 @@
       </c>
       <c r="L34" s="69"/>
     </row>
-    <row r="35" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="77" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D35" s="78" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E35" s="79" t="s">
         <v>91</v>
       </c>
       <c r="F35" s="78" t="s">
-        <v>152</v>
-      </c>
-      <c r="G35" s="107" t="s">
-        <v>378</v>
+        <v>151</v>
+      </c>
+      <c r="G35" s="78" t="s">
+        <v>377</v>
       </c>
       <c r="H35" s="78" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I35" s="79" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J35" s="80">
         <v>8</v>
@@ -3575,18 +3541,18 @@
         <v>160</v>
       </c>
       <c r="L35" s="74" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="O35" s="99"/>
     </row>
-    <row r="36" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C36" s="87" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D36" s="88" t="s">
         <v>23</v>
@@ -3595,16 +3561,16 @@
         <v>92</v>
       </c>
       <c r="F36" s="88" t="s">
-        <v>296</v>
-      </c>
-      <c r="G36" s="108" t="s">
-        <v>379</v>
+        <v>295</v>
+      </c>
+      <c r="G36" s="88" t="s">
+        <v>378</v>
       </c>
       <c r="H36" s="88" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I36" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J36" s="88">
         <v>1</v>
@@ -3615,14 +3581,14 @@
       </c>
       <c r="L36" s="82"/>
     </row>
-    <row r="37" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
       <c r="C37" s="90" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D37" s="91" t="s">
         <v>24</v>
@@ -3631,16 +3597,16 @@
         <v>93</v>
       </c>
       <c r="F37" s="91" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G37" s="92" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H37" s="91" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I37" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J37" s="91">
         <v>4</v>
@@ -3651,14 +3617,14 @@
       </c>
       <c r="L37" s="93"/>
     </row>
-    <row r="38" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C38" s="87" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D38" s="88" t="s">
         <v>25</v>
@@ -3667,16 +3633,16 @@
         <v>94</v>
       </c>
       <c r="F38" s="88" t="s">
-        <v>296</v>
-      </c>
-      <c r="G38" s="109" t="s">
-        <v>380</v>
+        <v>295</v>
+      </c>
+      <c r="G38" s="88" t="s">
+        <v>379</v>
       </c>
       <c r="H38" s="88" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I38" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J38" s="88">
         <v>1</v>
@@ -3687,14 +3653,14 @@
       </c>
       <c r="L38" s="69"/>
     </row>
-    <row r="39" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="53">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
       <c r="C39" s="90" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D39" s="91" t="s">
         <v>26</v>
@@ -3703,16 +3669,16 @@
         <v>95</v>
       </c>
       <c r="F39" s="91" t="s">
-        <v>296</v>
-      </c>
-      <c r="G39" s="110" t="s">
-        <v>381</v>
+        <v>295</v>
+      </c>
+      <c r="G39" s="91" t="s">
+        <v>380</v>
       </c>
       <c r="H39" s="91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I39" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J39" s="91">
         <v>2</v>
@@ -3723,14 +3689,14 @@
       </c>
       <c r="L39" s="70"/>
     </row>
-    <row r="40" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C40" s="87" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D40" s="88" t="s">
         <v>27</v>
@@ -3739,16 +3705,16 @@
         <v>96</v>
       </c>
       <c r="F40" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G40" s="89" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H40" s="88" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I40" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J40" s="88">
         <v>1</v>
@@ -3759,14 +3725,14 @@
       </c>
       <c r="L40" s="82"/>
     </row>
-    <row r="41" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
       <c r="C41" s="90" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D41" s="91" t="s">
         <v>28</v>
@@ -3775,16 +3741,16 @@
         <v>97</v>
       </c>
       <c r="F41" s="91" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G41" s="92" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H41" s="91" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I41" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J41" s="91">
         <v>1</v>
@@ -3795,29 +3761,29 @@
       </c>
       <c r="L41" s="93"/>
     </row>
-    <row r="42" spans="1:15" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:15" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="53"/>
       <c r="C42" s="90" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D42" s="91" t="s">
+        <v>370</v>
+      </c>
+      <c r="E42" s="92" t="s">
+        <v>372</v>
+      </c>
+      <c r="F42" s="91" t="s">
+        <v>295</v>
+      </c>
+      <c r="G42" s="92" t="s">
         <v>371</v>
       </c>
-      <c r="E42" s="92" t="s">
+      <c r="H42" s="91" t="s">
         <v>373</v>
       </c>
-      <c r="F42" s="91" t="s">
-        <v>296</v>
-      </c>
-      <c r="G42" s="92" t="s">
-        <v>372</v>
-      </c>
-      <c r="H42" s="91" t="s">
-        <v>374</v>
-      </c>
       <c r="I42" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J42" s="91">
         <v>1</v>
@@ -3828,14 +3794,14 @@
       </c>
       <c r="L42" s="93"/>
     </row>
-    <row r="43" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="53">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C43" s="87" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D43" s="88" t="s">
         <v>29</v>
@@ -3844,16 +3810,16 @@
         <v>98</v>
       </c>
       <c r="F43" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G43" s="89" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H43" s="88" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I43" s="89" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J43" s="88">
         <v>1</v>
@@ -3864,32 +3830,32 @@
       </c>
       <c r="L43" s="82"/>
     </row>
-    <row r="44" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="53">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
       <c r="C44" s="90" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D44" s="91" t="s">
         <v>30</v>
       </c>
       <c r="E44" s="92" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F44" s="91" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G44" s="92" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H44" s="91" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="I44" s="92" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="J44" s="91">
         <v>1</v>
@@ -3900,14 +3866,14 @@
       </c>
       <c r="L44" s="68"/>
     </row>
-    <row r="45" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="53">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C45" s="87" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D45" s="88" t="s">
         <v>31</v>
@@ -3916,16 +3882,16 @@
         <v>99</v>
       </c>
       <c r="F45" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G45" s="89" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H45" s="88" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I45" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J45" s="88">
         <v>1</v>
@@ -3936,14 +3902,14 @@
       </c>
       <c r="L45" s="82"/>
     </row>
-    <row r="46" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="53">
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
       <c r="C46" s="90" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D46" s="91" t="s">
         <v>32</v>
@@ -3952,16 +3918,16 @@
         <v>100</v>
       </c>
       <c r="F46" s="91" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G46" s="92" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H46" s="91" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I46" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J46" s="91">
         <v>1</v>
@@ -3972,32 +3938,32 @@
       </c>
       <c r="L46" s="93"/>
     </row>
-    <row r="47" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="53">
         <f t="shared" ref="B47:B90" si="2">ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
       <c r="C47" s="90" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D47" s="91" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E47" s="92" t="s">
+        <v>363</v>
+      </c>
+      <c r="F47" s="91" t="s">
+        <v>295</v>
+      </c>
+      <c r="G47" s="92" t="s">
         <v>364</v>
       </c>
-      <c r="F47" s="91" t="s">
-        <v>296</v>
-      </c>
-      <c r="G47" s="92" t="s">
+      <c r="H47" s="91" t="s">
         <v>365</v>
       </c>
-      <c r="H47" s="91" t="s">
-        <v>366</v>
-      </c>
       <c r="I47" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J47" s="91">
         <v>1</v>
@@ -4007,17 +3973,17 @@
         <v>20</v>
       </c>
       <c r="L47" s="70" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="53">
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
       <c r="C48" s="87" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D48" s="88" t="s">
         <v>33</v>
@@ -4026,16 +3992,16 @@
         <v>101</v>
       </c>
       <c r="F48" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G48" s="89" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H48" s="88" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I48" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J48" s="88">
         <v>2</v>
@@ -4046,14 +4012,14 @@
       </c>
       <c r="L48" s="82"/>
     </row>
-    <row r="49" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="53">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
       <c r="C49" s="83" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D49" s="84" t="s">
         <v>34</v>
@@ -4062,16 +4028,16 @@
         <v>102</v>
       </c>
       <c r="F49" s="84" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G49" s="85" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H49" s="84" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I49" s="85" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J49" s="84">
         <v>4</v>
@@ -4081,17 +4047,17 @@
         <v>80</v>
       </c>
       <c r="L49" s="62" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="53">
         <f t="shared" si="2"/>
         <v>41</v>
       </c>
       <c r="C50" s="87" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D50" s="88" t="s">
         <v>35</v>
@@ -4100,16 +4066,16 @@
         <v>103</v>
       </c>
       <c r="F50" s="88" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G50" s="89">
         <v>61300211121</v>
       </c>
       <c r="H50" s="88" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I50" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J50" s="88">
         <v>4</v>
@@ -4120,32 +4086,32 @@
       </c>
       <c r="L50" s="82"/>
     </row>
-    <row r="51" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="53">
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
       <c r="C51" s="90" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D51" s="91" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E51" s="92" t="s">
         <v>104</v>
       </c>
       <c r="F51" s="91" t="s">
-        <v>162</v>
-      </c>
-      <c r="G51" s="111" t="s">
-        <v>382</v>
+        <v>161</v>
+      </c>
+      <c r="G51" s="91" t="s">
+        <v>381</v>
       </c>
       <c r="H51" s="91" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I51" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J51" s="91">
         <v>4</v>
@@ -4156,14 +4122,14 @@
       </c>
       <c r="L51" s="93"/>
     </row>
-    <row r="52" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="53">
         <f t="shared" si="2"/>
         <v>43</v>
       </c>
       <c r="C52" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D52" s="88" t="s">
         <v>36</v>
@@ -4172,16 +4138,16 @@
         <v>105</v>
       </c>
       <c r="F52" s="88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G52" s="89" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H52" s="88" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I52" s="89" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J52" s="88">
         <v>2</v>
@@ -4192,14 +4158,14 @@
       </c>
       <c r="L52" s="82"/>
     </row>
-    <row r="53" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="53">
         <f t="shared" si="2"/>
         <v>44</v>
       </c>
       <c r="C53" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D53" s="91" t="s">
         <v>37</v>
@@ -4208,16 +4174,16 @@
         <v>106</v>
       </c>
       <c r="F53" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G53" s="92" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H53" s="91" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I53" s="92" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J53" s="91">
         <v>1</v>
@@ -4228,14 +4194,14 @@
       </c>
       <c r="L53" s="93"/>
     </row>
-    <row r="54" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="53">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="C54" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D54" s="88" t="s">
         <v>38</v>
@@ -4244,16 +4210,16 @@
         <v>107</v>
       </c>
       <c r="F54" s="88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G54" s="89" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H54" s="88" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I54" s="89" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J54" s="88">
         <v>1</v>
@@ -4264,14 +4230,14 @@
       </c>
       <c r="L54" s="82"/>
     </row>
-    <row r="55" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="53">
         <f t="shared" si="2"/>
         <v>46</v>
       </c>
       <c r="C55" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D55" s="91" t="s">
         <v>39</v>
@@ -4280,16 +4246,16 @@
         <v>108</v>
       </c>
       <c r="F55" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G55" s="92" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H55" s="91" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I55" s="92" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J55" s="91">
         <v>2</v>
@@ -4300,14 +4266,14 @@
       </c>
       <c r="L55" s="93"/>
     </row>
-    <row r="56" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="53">
         <f t="shared" si="2"/>
         <v>47</v>
       </c>
       <c r="C56" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D56" s="88" t="s">
         <v>40</v>
@@ -4316,16 +4282,16 @@
         <v>109</v>
       </c>
       <c r="F56" s="88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G56" s="89" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H56" s="88" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I56" s="89" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J56" s="88">
         <v>4</v>
@@ -4336,14 +4302,14 @@
       </c>
       <c r="L56" s="82"/>
     </row>
-    <row r="57" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="53">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
       <c r="C57" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D57" s="91" t="s">
         <v>41</v>
@@ -4352,16 +4318,16 @@
         <v>110</v>
       </c>
       <c r="F57" s="91" t="s">
-        <v>164</v>
-      </c>
-      <c r="G57" s="112" t="s">
-        <v>383</v>
+        <v>163</v>
+      </c>
+      <c r="G57" s="91" t="s">
+        <v>382</v>
       </c>
       <c r="H57" s="91" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I57" s="92" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J57" s="91">
         <v>4</v>
@@ -4372,32 +4338,32 @@
       </c>
       <c r="L57" s="93"/>
     </row>
-    <row r="58" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="53">
         <f t="shared" si="2"/>
         <v>49</v>
       </c>
       <c r="C58" s="60" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D58" s="37" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E58" s="37" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G58" s="37" t="s">
+        <v>326</v>
+      </c>
+      <c r="H58" s="37" t="s">
+        <v>239</v>
+      </c>
+      <c r="I58" s="37" t="s">
         <v>327</v>
-      </c>
-      <c r="H58" s="37" t="s">
-        <v>240</v>
-      </c>
-      <c r="I58" s="37" t="s">
-        <v>328</v>
       </c>
       <c r="J58" s="37">
         <v>8</v>
@@ -4408,14 +4374,14 @@
       </c>
       <c r="L58" s="67"/>
     </row>
-    <row r="59" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="53">
         <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="C59" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D59" s="91" t="s">
         <v>42</v>
@@ -4424,16 +4390,16 @@
         <v>112</v>
       </c>
       <c r="F59" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G59" s="92" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H59" s="91" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I59" s="92" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J59" s="91">
         <v>1</v>
@@ -4444,14 +4410,14 @@
       </c>
       <c r="L59" s="93"/>
     </row>
-    <row r="60" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="53">
         <f t="shared" si="2"/>
         <v>51</v>
       </c>
       <c r="C60" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D60" s="88" t="s">
         <v>43</v>
@@ -4460,16 +4426,16 @@
         <v>113</v>
       </c>
       <c r="F60" s="88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G60" s="89" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H60" s="88" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I60" s="89" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J60" s="88">
         <v>1</v>
@@ -4480,14 +4446,14 @@
       </c>
       <c r="L60" s="82"/>
     </row>
-    <row r="61" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="53">
         <f t="shared" si="2"/>
         <v>52</v>
       </c>
       <c r="C61" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D61" s="91" t="s">
         <v>44</v>
@@ -4496,16 +4462,16 @@
         <v>114</v>
       </c>
       <c r="F61" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G61" s="92" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H61" s="91" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I61" s="92" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J61" s="91">
         <v>1</v>
@@ -4516,14 +4482,14 @@
       </c>
       <c r="L61" s="93"/>
     </row>
-    <row r="62" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="53">
         <f t="shared" si="2"/>
         <v>53</v>
       </c>
       <c r="C62" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D62" s="88" t="s">
         <v>45</v>
@@ -4532,16 +4498,16 @@
         <v>115</v>
       </c>
       <c r="F62" s="88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G62" s="89" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H62" s="88" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I62" s="89" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J62" s="88">
         <v>1</v>
@@ -4552,14 +4518,14 @@
       </c>
       <c r="L62" s="82"/>
     </row>
-    <row r="63" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="53">
         <f t="shared" si="2"/>
         <v>54</v>
       </c>
       <c r="C63" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D63" s="91" t="s">
         <v>46</v>
@@ -4568,16 +4534,16 @@
         <v>116</v>
       </c>
       <c r="F63" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G63" s="92" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H63" s="91" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I63" s="92" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J63" s="91">
         <v>1</v>
@@ -4588,14 +4554,14 @@
       </c>
       <c r="L63" s="93"/>
     </row>
-    <row r="64" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="53">
         <f t="shared" si="2"/>
         <v>55</v>
       </c>
       <c r="C64" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D64" s="88" t="s">
         <v>47</v>
@@ -4604,16 +4570,16 @@
         <v>117</v>
       </c>
       <c r="F64" s="88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G64" s="89" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H64" s="88" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I64" s="89" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J64" s="88">
         <v>1</v>
@@ -4624,14 +4590,14 @@
       </c>
       <c r="L64" s="82"/>
     </row>
-    <row r="65" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="53">
         <f t="shared" si="2"/>
         <v>56</v>
       </c>
       <c r="C65" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D65" s="91" t="s">
         <v>48</v>
@@ -4640,16 +4606,16 @@
         <v>118</v>
       </c>
       <c r="F65" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G65" s="92" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H65" s="91" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I65" s="92" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="J65" s="91">
         <v>1</v>
@@ -4660,14 +4626,14 @@
       </c>
       <c r="L65" s="93"/>
     </row>
-    <row r="66" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="53">
         <f t="shared" si="2"/>
         <v>57</v>
       </c>
       <c r="C66" s="87" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D66" s="88" t="s">
         <v>49</v>
@@ -4676,16 +4642,16 @@
         <v>119</v>
       </c>
       <c r="F66" s="88" t="s">
-        <v>163</v>
-      </c>
-      <c r="G66" s="113" t="s">
-        <v>384</v>
+        <v>162</v>
+      </c>
+      <c r="G66" s="88" t="s">
+        <v>383</v>
       </c>
       <c r="H66" s="88" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I66" s="89" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J66" s="88">
         <v>1</v>
@@ -4696,32 +4662,32 @@
       </c>
       <c r="L66" s="82"/>
     </row>
-    <row r="67" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="53">
         <f t="shared" si="2"/>
         <v>58</v>
       </c>
       <c r="C67" s="90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D67" s="91" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E67" s="92" t="s">
         <v>120</v>
       </c>
       <c r="F67" s="91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G67" s="92" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H67" s="91" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I67" s="92" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J67" s="91">
         <v>2</v>
@@ -4732,14 +4698,14 @@
       </c>
       <c r="L67" s="93"/>
     </row>
-    <row r="68" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="53">
         <f t="shared" si="2"/>
         <v>59</v>
       </c>
       <c r="C68" s="60" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D68" s="37" t="s">
         <v>50</v>
@@ -4748,16 +4714,16 @@
         <v>121</v>
       </c>
       <c r="F68" s="37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H68" s="37" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I68" s="38" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J68" s="37">
         <v>2</v>
@@ -4768,32 +4734,32 @@
       </c>
       <c r="L68" s="41"/>
     </row>
-    <row r="69" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="53">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
       <c r="C69" s="59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D69" s="76" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E69" s="40" t="s">
         <v>111</v>
       </c>
       <c r="F69" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G69" s="40" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H69" s="39" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I69" s="40" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J69" s="39">
         <v>1</v>
@@ -4804,14 +4770,14 @@
       </c>
       <c r="L69" s="68"/>
     </row>
-    <row r="70" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="53">
         <f t="shared" si="2"/>
         <v>61</v>
       </c>
       <c r="C70" s="60" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D70" s="37" t="s">
         <v>51</v>
@@ -4820,16 +4786,16 @@
         <v>122</v>
       </c>
       <c r="F70" s="37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G70" s="38" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H70" s="37" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I70" s="38" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J70" s="37">
         <v>2</v>
@@ -4840,14 +4806,14 @@
       </c>
       <c r="L70" s="41"/>
     </row>
-    <row r="71" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="53">
         <f t="shared" si="2"/>
         <v>62</v>
       </c>
       <c r="C71" s="59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D71" s="39" t="s">
         <v>52</v>
@@ -4856,16 +4822,16 @@
         <v>123</v>
       </c>
       <c r="F71" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G71" s="40" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H71" s="39" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I71" s="40" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J71" s="39">
         <v>1</v>
@@ -4876,32 +4842,32 @@
       </c>
       <c r="L71" s="42"/>
     </row>
-    <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="53">
         <f t="shared" si="2"/>
         <v>63</v>
       </c>
       <c r="C72" s="60" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D72" s="37" t="s">
         <v>53</v>
       </c>
       <c r="E72" s="38" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F72" s="75" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G72" s="38" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H72" s="37" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I72" s="38" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J72" s="37">
         <v>1</v>
@@ -4912,32 +4878,32 @@
       </c>
       <c r="L72" s="67"/>
     </row>
-    <row r="73" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="53">
         <f t="shared" si="2"/>
         <v>64</v>
       </c>
       <c r="C73" s="59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D73" s="39" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E73" s="40" t="s">
         <v>127</v>
       </c>
       <c r="F73" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G73" s="40" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H73" s="39" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I73" s="40" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J73" s="39">
         <v>6</v>
@@ -4948,14 +4914,14 @@
       </c>
       <c r="L73" s="68"/>
     </row>
-    <row r="74" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="53">
         <f t="shared" si="2"/>
         <v>65</v>
       </c>
       <c r="C74" s="60" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D74" s="37" t="s">
         <v>54</v>
@@ -4964,16 +4930,16 @@
         <v>124</v>
       </c>
       <c r="F74" s="37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G74" s="38" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H74" s="37" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I74" s="38" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J74" s="37">
         <v>1</v>
@@ -4984,14 +4950,14 @@
       </c>
       <c r="L74" s="41"/>
     </row>
-    <row r="75" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="53">
         <f t="shared" si="2"/>
         <v>66</v>
       </c>
       <c r="C75" s="59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D75" s="39" t="s">
         <v>55</v>
@@ -5000,16 +4966,16 @@
         <v>125</v>
       </c>
       <c r="F75" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G75" s="40" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H75" s="39" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I75" s="40" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J75" s="39">
         <v>1</v>
@@ -5020,14 +4986,14 @@
       </c>
       <c r="L75" s="42"/>
     </row>
-    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="53">
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
       <c r="C76" s="83" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D76" s="84" t="s">
         <v>56</v>
@@ -5036,16 +5002,16 @@
         <v>126</v>
       </c>
       <c r="F76" s="84" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G76" s="85" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H76" s="84" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I76" s="85" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J76" s="84">
         <v>4</v>
@@ -5055,35 +5021,35 @@
         <v>80</v>
       </c>
       <c r="L76" s="62" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="53">
         <f t="shared" si="2"/>
         <v>68</v>
       </c>
       <c r="C77" s="83" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D77" s="84" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E77" s="85" t="s">
         <v>128</v>
       </c>
       <c r="F77" s="84" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G77" s="85" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H77" s="84" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I77" s="85" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J77" s="84">
         <v>15</v>
@@ -5093,17 +5059,17 @@
         <v>300</v>
       </c>
       <c r="L77" s="62" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="53">
         <f t="shared" si="2"/>
         <v>69</v>
       </c>
       <c r="C78" s="87" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D78" s="88" t="s">
         <v>57</v>
@@ -5112,16 +5078,16 @@
         <v>129</v>
       </c>
       <c r="F78" s="88" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G78" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H78" s="88" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I78" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J78" s="88">
         <v>1</v>
@@ -5132,14 +5098,14 @@
       </c>
       <c r="L78" s="82"/>
     </row>
-    <row r="79" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="53">
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
       <c r="C79" s="90" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D79" s="91" t="s">
         <v>58</v>
@@ -5148,16 +5114,16 @@
         <v>130</v>
       </c>
       <c r="F79" s="91" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G79" s="92">
         <v>750314597</v>
       </c>
       <c r="H79" s="91" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I79" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J79" s="91">
         <v>1</v>
@@ -5168,14 +5134,14 @@
       </c>
       <c r="L79" s="93"/>
     </row>
-    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="53">
         <f t="shared" si="2"/>
         <v>71</v>
       </c>
       <c r="C80" s="87" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D80" s="88" t="s">
         <v>59</v>
@@ -5184,16 +5150,16 @@
         <v>131</v>
       </c>
       <c r="F80" s="88" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G80" s="89" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H80" s="88" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I80" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J80" s="88">
         <v>1</v>
@@ -5204,14 +5170,14 @@
       </c>
       <c r="L80" s="82"/>
     </row>
-    <row r="81" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="53">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="C81" s="90" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D81" s="91" t="s">
         <v>60</v>
@@ -5220,16 +5186,16 @@
         <v>132</v>
       </c>
       <c r="F81" s="91" t="s">
-        <v>169</v>
-      </c>
-      <c r="G81" s="114" t="s">
-        <v>385</v>
+        <v>168</v>
+      </c>
+      <c r="G81" s="91" t="s">
+        <v>384</v>
       </c>
       <c r="H81" s="91" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I81" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J81" s="91">
         <v>1</v>
@@ -5240,14 +5206,14 @@
       </c>
       <c r="L81" s="70"/>
     </row>
-    <row r="82" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="53">
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
       <c r="C82" s="87" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D82" s="88" t="s">
         <v>61</v>
@@ -5256,16 +5222,16 @@
         <v>133</v>
       </c>
       <c r="F82" s="88" t="s">
-        <v>170</v>
-      </c>
-      <c r="G82" s="115" t="s">
-        <v>386</v>
+        <v>169</v>
+      </c>
+      <c r="G82" s="88" t="s">
+        <v>385</v>
       </c>
       <c r="H82" s="88" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I82" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J82" s="88">
         <v>1</v>
@@ -5276,14 +5242,14 @@
       </c>
       <c r="L82" s="69"/>
     </row>
-    <row r="83" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="53">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
       <c r="C83" s="90" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D83" s="91" t="s">
         <v>62</v>
@@ -5292,16 +5258,16 @@
         <v>134</v>
       </c>
       <c r="F83" s="91" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G83" s="92" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H83" s="91" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I83" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J83" s="91">
         <v>1</v>
@@ -5312,14 +5278,14 @@
       </c>
       <c r="L83" s="93"/>
     </row>
-    <row r="84" spans="1:15" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:15" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
       <c r="B84" s="53">
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
       <c r="C84" s="87" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D84" s="88" t="s">
         <v>63</v>
@@ -5328,16 +5294,16 @@
         <v>135</v>
       </c>
       <c r="F84" s="88" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G84" s="89" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H84" s="88" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I84" s="89" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J84" s="88">
         <v>1</v>
@@ -5348,14 +5314,14 @@
       </c>
       <c r="L84" s="82"/>
     </row>
-    <row r="85" spans="1:15" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:15" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="53">
         <f t="shared" si="2"/>
         <v>76</v>
       </c>
       <c r="C85" s="63" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D85" s="64" t="s">
         <v>64</v>
@@ -5364,16 +5330,16 @@
         <v>136</v>
       </c>
       <c r="F85" s="64" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G85" s="65" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H85" s="64" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I85" s="65" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J85" s="64">
         <v>1</v>
@@ -5383,18 +5349,18 @@
         <v>20</v>
       </c>
       <c r="L85" s="66" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="O85" s="98"/>
     </row>
-    <row r="86" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="53">
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
       <c r="C86" s="87" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D86" s="88" t="s">
         <v>65</v>
@@ -5403,16 +5369,16 @@
         <v>137</v>
       </c>
       <c r="F86" s="88" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G86" s="89" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H86" s="88" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I86" s="96" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J86" s="88">
         <v>1</v>
@@ -5423,32 +5389,32 @@
       </c>
       <c r="L86" s="82"/>
     </row>
-    <row r="87" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
       <c r="B87" s="53">
         <f t="shared" si="2"/>
         <v>78</v>
       </c>
       <c r="C87" s="90" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D87" s="91" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E87" s="92" t="s">
         <v>138</v>
       </c>
       <c r="F87" s="91" t="s">
-        <v>299</v>
-      </c>
-      <c r="G87" s="116" t="s">
-        <v>387</v>
+        <v>298</v>
+      </c>
+      <c r="G87" s="91" t="s">
+        <v>386</v>
       </c>
       <c r="H87" s="91" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I87" s="92" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J87" s="97">
         <v>2</v>
@@ -5459,14 +5425,14 @@
       </c>
       <c r="L87" s="70"/>
     </row>
-    <row r="88" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="53">
         <f t="shared" si="2"/>
         <v>79</v>
       </c>
       <c r="C88" s="60" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D88" s="37" t="s">
         <v>66</v>
@@ -5475,16 +5441,16 @@
         <v>140</v>
       </c>
       <c r="F88" s="37" t="s">
+        <v>300</v>
+      </c>
+      <c r="G88" s="38" t="s">
+        <v>174</v>
+      </c>
+      <c r="H88" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="I88" s="38" t="s">
         <v>301</v>
-      </c>
-      <c r="G88" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="H88" s="37" t="s">
-        <v>244</v>
-      </c>
-      <c r="I88" s="38" t="s">
-        <v>302</v>
       </c>
       <c r="J88" s="37">
         <v>1</v>
@@ -5495,32 +5461,32 @@
       </c>
       <c r="L88" s="41"/>
     </row>
-    <row r="89" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
       <c r="B89" s="53">
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
       <c r="C89" s="59" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D89" s="39" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E89" s="40" t="s">
         <v>139</v>
       </c>
       <c r="F89" s="39" t="s">
-        <v>300</v>
-      </c>
-      <c r="G89" s="117" t="s">
-        <v>388</v>
+        <v>299</v>
+      </c>
+      <c r="G89" s="39" t="s">
+        <v>387</v>
       </c>
       <c r="H89" s="39" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I89" s="40" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J89" s="39">
         <v>1</v>
@@ -5531,29 +5497,29 @@
       </c>
       <c r="L89" s="70"/>
     </row>
-    <row r="90" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
       <c r="B90" s="53">
         <f t="shared" si="2"/>
         <v>81</v>
       </c>
       <c r="C90" s="59" t="s">
+        <v>366</v>
+      </c>
+      <c r="D90" s="39" t="s">
+        <v>301</v>
+      </c>
+      <c r="E90" s="40" t="s">
+        <v>369</v>
+      </c>
+      <c r="F90" s="39" t="s">
+        <v>295</v>
+      </c>
+      <c r="G90" s="40" t="s">
         <v>367</v>
       </c>
-      <c r="D90" s="39" t="s">
-        <v>302</v>
-      </c>
-      <c r="E90" s="40" t="s">
-        <v>370</v>
-      </c>
-      <c r="F90" s="39" t="s">
-        <v>296</v>
-      </c>
-      <c r="G90" s="40" t="s">
+      <c r="H90" s="39" t="s">
         <v>368</v>
-      </c>
-      <c r="H90" s="39" t="s">
-        <v>369</v>
       </c>
       <c r="I90" s="40"/>
       <c r="J90" s="39">
@@ -5565,7 +5531,7 @@
       </c>
       <c r="L90" s="70"/>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="32"/>
       <c r="C91" s="51"/>
@@ -5581,7 +5547,7 @@
       <c r="K91" s="36"/>
       <c r="L91" s="44"/>
     </row>
-    <row r="92" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="1"/>
       <c r="B92" s="24"/>
       <c r="C92" s="52"/>

</xml_diff>